<commit_message>
Actualizar datos con datos 4.xlsx (incluye Retail)
Se publica el Excel "datos 4.xlsx" renombrado a datos.xlsx, con Retail en
Negocio_Volumen y Negocio_Horas, entrega de Retail hasta septiembre y un
freelance más en septiembre.

La hoja Ciudad se mantiene como estaba publicada: en la nueva, Madrid
febrero vale 73208 (falta "=" y "+") y las sumas añadidas a Madrid hacen
que las ciudades sumen el doble que el total de trabajos. Queda
pendiente de que se corrija en el Excel.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01A4SLDFHLc22bTWoXT2NUrv
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Instrucciones" sheetId="1" state="visible" r:id="rId3"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="119">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="219" uniqueCount="119">
   <si>
     <t xml:space="preserve">PLANTILLA DASHBOARD BDESIGN</t>
   </si>
@@ -332,6 +332,9 @@
     <t xml:space="preserve">Foro Innovacion</t>
   </si>
   <si>
+    <t xml:space="preserve">Retail</t>
+  </si>
+  <si>
     <t xml:space="preserve">HORAS dedicadas por DEPARTAMENTO/NEGOCIO</t>
   </si>
   <si>
@@ -363,9 +366,6 @@
   </si>
   <si>
     <t xml:space="preserve">Bdesign</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Retail</t>
   </si>
   <si>
     <t xml:space="preserve">MEDIA YTD</t>
@@ -395,7 +395,7 @@
     <numFmt numFmtId="165" formatCode="General"/>
     <numFmt numFmtId="166" formatCode="0.0"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="14">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -471,6 +471,21 @@
       <charset val="1"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
@@ -492,7 +507,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
@@ -512,6 +527,21 @@
       </top>
       <bottom style="thin">
         <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="medium">
+        <color rgb="FFE6E6E6"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFE6E6E6"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFE6E6E6"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFE6E6E6"/>
       </bottom>
       <diagonal/>
     </border>
@@ -541,7 +571,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="19">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -586,12 +616,28 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
@@ -631,7 +677,7 @@
       <rgbColor rgb="FF808080"/>
       <rgbColor rgb="FF9999FF"/>
       <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FFFFFFCC"/>
+      <rgbColor rgb="FFE6E6E6"/>
       <rgbColor rgb="FFCCFFFF"/>
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
@@ -855,7 +901,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D37"/>
-  <sheetFormatPr defaultColWidth="8.66796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.66796875" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="24"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="2" style="0" width="28"/>
@@ -1151,7 +1197,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:L19"/>
-  <sheetFormatPr defaultColWidth="8.66796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.66796875" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="2" style="0" width="14"/>
@@ -1173,7 +1219,7 @@
       <c r="K1" s="10"/>
       <c r="L1" s="10"/>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
         <v>48</v>
       </c>
@@ -1211,57 +1257,57 @@
         <v>59</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="11" t="s">
         <v>60</v>
       </c>
       <c r="B4" s="11" t="n">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="C4" s="11" t="n">
-        <v>28</v>
+        <v>40</v>
       </c>
       <c r="D4" s="11" t="n">
-        <v>23</v>
+        <v>32</v>
       </c>
       <c r="E4" s="11" t="n">
-        <v>25</v>
+        <v>34</v>
       </c>
       <c r="F4" s="11" t="n">
-        <v>36</v>
+        <v>45</v>
       </c>
       <c r="G4" s="11" t="n">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="H4" s="11" t="n">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="I4" s="11" t="n">
         <v>10</v>
       </c>
       <c r="J4" s="11" t="n">
-        <v>41</v>
+        <v>52</v>
       </c>
       <c r="K4" s="11" t="n">
-        <v>48</v>
-      </c>
-      <c r="L4" s="11" t="n">
+        <v>55</v>
+      </c>
+      <c r="L4" s="12" t="n">
         <f aca="false">SUM(B4:K4)</f>
-        <v>307</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="11" t="s">
         <v>45</v>
       </c>
       <c r="B5" s="11" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C5" s="11" t="n">
         <v>21</v>
       </c>
       <c r="D5" s="11" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E5" s="11" t="n">
         <v>7</v>
@@ -1270,26 +1316,26 @@
         <v>19</v>
       </c>
       <c r="G5" s="11" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="H5" s="11" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="I5" s="11" t="n">
         <v>7</v>
       </c>
       <c r="J5" s="11" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="K5" s="11" t="n">
-        <v>22</v>
-      </c>
-      <c r="L5" s="11" t="n">
+        <v>23</v>
+      </c>
+      <c r="L5" s="12" t="n">
         <f aca="false">SUM(B5:K5)</f>
-        <v>204</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="11" t="s">
         <v>61</v>
       </c>
@@ -1303,89 +1349,91 @@
         <v>12</v>
       </c>
       <c r="E6" s="11" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="F6" s="11" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="G6" s="11" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="H6" s="11" t="n">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="I6" s="11" t="n">
         <v>2</v>
       </c>
       <c r="J6" s="11" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="K6" s="11" t="n">
         <v>31</v>
       </c>
-      <c r="L6" s="11" t="n">
+      <c r="L6" s="12" t="n">
         <f aca="false">SUM(B6:K6)</f>
-        <v>175</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="11" t="s">
         <v>62</v>
       </c>
       <c r="B7" s="11" t="n">
+        <v>16</v>
+      </c>
+      <c r="C7" s="11" t="n">
         <v>14</v>
       </c>
-      <c r="C7" s="11" t="n">
-        <v>8</v>
-      </c>
       <c r="D7" s="11" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E7" s="11" t="n">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="F7" s="11" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="G7" s="11" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="H7" s="11" t="n">
-        <v>10</v>
-      </c>
-      <c r="I7" s="11"/>
+        <v>15</v>
+      </c>
+      <c r="I7" s="11" t="n">
+        <v>0</v>
+      </c>
       <c r="J7" s="11" t="n">
         <v>4</v>
       </c>
       <c r="K7" s="11" t="n">
-        <v>8</v>
-      </c>
-      <c r="L7" s="11" t="n">
+        <v>9</v>
+      </c>
+      <c r="L7" s="12" t="n">
         <f aca="false">SUM(B7:K7)</f>
-        <v>83</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="11" t="s">
         <v>63</v>
       </c>
       <c r="B8" s="11" t="n">
+        <v>11</v>
+      </c>
+      <c r="C8" s="11" t="n">
+        <v>7</v>
+      </c>
+      <c r="D8" s="11" t="n">
         <v>9</v>
-      </c>
-      <c r="C8" s="11" t="n">
-        <v>6</v>
-      </c>
-      <c r="D8" s="11" t="n">
-        <v>6</v>
       </c>
       <c r="E8" s="11" t="n">
         <v>10</v>
       </c>
       <c r="F8" s="11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G8" s="11" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="H8" s="11" t="n">
         <v>5</v>
@@ -1394,17 +1442,17 @@
         <v>3</v>
       </c>
       <c r="J8" s="11" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="K8" s="11" t="n">
-        <v>6</v>
-      </c>
-      <c r="L8" s="11" t="n">
+        <v>7</v>
+      </c>
+      <c r="L8" s="12" t="n">
         <f aca="false">SUM(B8:K8)</f>
-        <v>67</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="11" t="s">
         <v>64</v>
       </c>
@@ -1433,93 +1481,95 @@
         <v>2</v>
       </c>
       <c r="J9" s="11" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="K9" s="11" t="n">
         <v>5</v>
       </c>
-      <c r="L9" s="11" t="n">
+      <c r="L9" s="12" t="n">
         <f aca="false">SUM(B9:K9)</f>
-        <v>58</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="11" t="s">
         <v>65</v>
       </c>
       <c r="B10" s="11" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C10" s="11" t="n">
+        <v>9</v>
+      </c>
+      <c r="D10" s="11" t="n">
+        <v>7</v>
+      </c>
+      <c r="E10" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="D10" s="11" t="n">
+      <c r="F10" s="11" t="n">
         <v>6</v>
       </c>
-      <c r="E10" s="11" t="n">
+      <c r="G10" s="11" t="n">
         <v>6</v>
       </c>
-      <c r="F10" s="11" t="n">
-        <v>3</v>
-      </c>
-      <c r="G10" s="11" t="n">
-        <v>5</v>
-      </c>
       <c r="H10" s="11" t="n">
-        <v>11</v>
-      </c>
-      <c r="I10" s="11"/>
+        <v>13</v>
+      </c>
+      <c r="I10" s="11" t="n">
+        <v>0</v>
+      </c>
       <c r="J10" s="11" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="K10" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="L10" s="11" t="n">
+      <c r="L10" s="12" t="n">
         <f aca="false">SUM(B10:K10)</f>
-        <v>53</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="11" t="s">
         <v>66</v>
       </c>
       <c r="B11" s="11" t="n">
+        <v>10</v>
+      </c>
+      <c r="C11" s="11" t="n">
+        <v>10</v>
+      </c>
+      <c r="D11" s="11" t="n">
+        <v>7</v>
+      </c>
+      <c r="E11" s="11" t="n">
+        <v>5</v>
+      </c>
+      <c r="F11" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="G11" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="H11" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="I11" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="J11" s="11" t="n">
+        <v>11</v>
+      </c>
+      <c r="K11" s="11" t="n">
         <v>9</v>
       </c>
-      <c r="C11" s="11" t="n">
-        <v>4</v>
-      </c>
-      <c r="D11" s="11" t="n">
-        <v>4</v>
-      </c>
-      <c r="E11" s="11" t="n">
-        <v>3</v>
-      </c>
-      <c r="F11" s="11" t="n">
-        <v>3</v>
-      </c>
-      <c r="G11" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="H11" s="11" t="n">
-        <v>3</v>
-      </c>
-      <c r="I11" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="J11" s="11" t="n">
-        <v>7</v>
-      </c>
-      <c r="K11" s="11" t="n">
-        <v>3</v>
-      </c>
-      <c r="L11" s="11" t="n">
+      <c r="L11" s="12" t="n">
         <f aca="false">SUM(B11:K11)</f>
-        <v>40</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="11" t="s">
         <v>67</v>
       </c>
@@ -1529,8 +1579,12 @@
       <c r="C12" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="D12" s="11"/>
-      <c r="E12" s="11"/>
+      <c r="D12" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" s="11" t="n">
+        <v>0</v>
+      </c>
       <c r="F12" s="11" t="n">
         <v>7</v>
       </c>
@@ -1538,66 +1592,74 @@
         <v>4</v>
       </c>
       <c r="H12" s="11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I12" s="11" t="n">
         <v>2</v>
       </c>
       <c r="J12" s="11" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="K12" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="L12" s="11" t="n">
+      <c r="L12" s="12" t="n">
         <f aca="false">SUM(B12:K12)</f>
-        <v>26</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="11" t="s">
         <v>68</v>
       </c>
       <c r="B13" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="C13" s="11"/>
-      <c r="D13" s="11"/>
+      <c r="C13" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13" s="11" t="n">
+        <v>2</v>
+      </c>
       <c r="E13" s="11" t="n">
         <v>1</v>
       </c>
       <c r="F13" s="11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G13" s="11" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H13" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="I13" s="11"/>
+        <v>6</v>
+      </c>
+      <c r="I13" s="11" t="n">
+        <v>0</v>
+      </c>
       <c r="J13" s="11" t="n">
         <v>1</v>
       </c>
       <c r="K13" s="11" t="n">
         <v>6</v>
       </c>
-      <c r="L13" s="11" t="n">
+      <c r="L13" s="12" t="n">
         <f aca="false">SUM(B13:K13)</f>
-        <v>18</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="11" t="s">
         <v>69</v>
       </c>
       <c r="B14" s="11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C14" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="D14" s="11"/>
+      <c r="D14" s="11" t="n">
+        <v>0</v>
+      </c>
       <c r="E14" s="11" t="n">
         <v>3</v>
       </c>
@@ -1605,31 +1667,37 @@
         <v>2</v>
       </c>
       <c r="G14" s="11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H14" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="I14" s="11"/>
+      <c r="I14" s="11" t="n">
+        <v>0</v>
+      </c>
       <c r="J14" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="K14" s="11"/>
-      <c r="L14" s="11" t="n">
+      <c r="K14" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" s="12" t="n">
         <f aca="false">SUM(B14:K14)</f>
-        <v>16</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="11" t="s">
         <v>70</v>
       </c>
       <c r="B15" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="C15" s="11"/>
+      <c r="C15" s="11" t="n">
+        <v>0</v>
+      </c>
       <c r="D15" s="11" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E15" s="11" t="n">
         <v>2</v>
@@ -1638,62 +1706,86 @@
         <v>1</v>
       </c>
       <c r="G15" s="11" t="n">
-        <v>4</v>
-      </c>
-      <c r="H15" s="11"/>
-      <c r="I15" s="11"/>
-      <c r="J15" s="11"/>
+        <v>5</v>
+      </c>
+      <c r="H15" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J15" s="11" t="n">
+        <v>0</v>
+      </c>
       <c r="K15" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="L15" s="11" t="n">
+      <c r="L15" s="12" t="n">
         <f aca="false">SUM(B15:K15)</f>
-        <v>14</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="11" t="s">
         <v>71</v>
       </c>
       <c r="B16" s="11" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C16" s="11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D16" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="E16" s="11"/>
-      <c r="F16" s="11"/>
+        <v>4</v>
+      </c>
+      <c r="E16" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F16" s="11" t="n">
+        <v>0</v>
+      </c>
       <c r="G16" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="H16" s="11"/>
+        <v>2</v>
+      </c>
+      <c r="H16" s="11" t="n">
+        <v>0</v>
+      </c>
       <c r="I16" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="J16" s="11"/>
+      <c r="J16" s="11" t="n">
+        <v>3</v>
+      </c>
       <c r="K16" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="L16" s="11" t="n">
+      <c r="L16" s="12" t="n">
         <f aca="false">SUM(B16:K16)</f>
-        <v>10</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="11" t="s">
         <v>72</v>
       </c>
-      <c r="B17" s="11"/>
-      <c r="C17" s="11"/>
-      <c r="D17" s="11"/>
+      <c r="B17" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D17" s="11" t="n">
+        <v>1</v>
+      </c>
       <c r="E17" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="F17" s="11"/>
-      <c r="G17" s="11"/>
+      <c r="F17" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" s="11" t="n">
+        <v>2</v>
+      </c>
       <c r="H17" s="11" t="n">
         <v>1</v>
       </c>
@@ -1703,84 +1795,97 @@
       <c r="J17" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="K17" s="11"/>
-      <c r="L17" s="11" t="n">
+      <c r="K17" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="L17" s="12" t="n">
         <f aca="false">SUM(B17:K17)</f>
-        <v>5</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="11" t="s">
         <v>73</v>
       </c>
-      <c r="B18" s="11"/>
-      <c r="C18" s="11"/>
-      <c r="D18" s="11"/>
-      <c r="E18" s="11"/>
+      <c r="B18" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="C18" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D18" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E18" s="11" t="n">
+        <v>0</v>
+      </c>
       <c r="F18" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="G18" s="11"/>
-      <c r="H18" s="11"/>
-      <c r="I18" s="11"/>
+        <v>3</v>
+      </c>
+      <c r="G18" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="I18" s="11" t="n">
+        <v>0</v>
+      </c>
       <c r="J18" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="K18" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="L18" s="11" t="n">
+      <c r="L18" s="12" t="n">
         <f aca="false">SUM(B18:K18)</f>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="s">
         <v>74</v>
       </c>
-      <c r="B19" s="12" t="n">
+      <c r="B19" s="13" t="n">
         <f aca="false">SUM(B4:B18)</f>
-        <v>112</v>
-      </c>
-      <c r="C19" s="12" t="n">
+        <v>130</v>
+      </c>
+      <c r="C19" s="13" t="n">
         <f aca="false">SUM(C4:C18)</f>
-        <v>107</v>
-      </c>
-      <c r="D19" s="12" t="n">
+        <v>134</v>
+      </c>
+      <c r="D19" s="13" t="n">
         <f aca="false">SUM(D4:D18)</f>
-        <v>91</v>
-      </c>
-      <c r="E19" s="12" t="n">
+        <v>118</v>
+      </c>
+      <c r="E19" s="13" t="n">
         <f aca="false">SUM(E4:E18)</f>
-        <v>88</v>
-      </c>
-      <c r="F19" s="12" t="n">
+        <v>114</v>
+      </c>
+      <c r="F19" s="13" t="n">
         <f aca="false">SUM(F4:F18)</f>
-        <v>114</v>
-      </c>
-      <c r="G19" s="12" t="n">
+        <v>136</v>
+      </c>
+      <c r="G19" s="13" t="n">
         <f aca="false">SUM(G4:G18)</f>
-        <v>150</v>
-      </c>
-      <c r="H19" s="12" t="n">
+        <v>177</v>
+      </c>
+      <c r="H19" s="13" t="n">
         <f aca="false">SUM(H4:H18)</f>
-        <v>136</v>
-      </c>
-      <c r="I19" s="12" t="n">
+        <v>163</v>
+      </c>
+      <c r="I19" s="13" t="n">
         <f aca="false">SUM(I4:I18)</f>
         <v>30</v>
       </c>
-      <c r="J19" s="12" t="n">
+      <c r="J19" s="13" t="n">
         <f aca="false">SUM(J4:J18)</f>
-        <v>112</v>
-      </c>
-      <c r="K19" s="12" t="n">
+        <v>145</v>
+      </c>
+      <c r="K19" s="13" t="n">
         <f aca="false">SUM(K4:K18)</f>
-        <v>139</v>
-      </c>
-      <c r="L19" s="12" t="n">
+        <v>154</v>
+      </c>
+      <c r="L19" s="13" t="n">
         <f aca="false">SUM(L4:L18)</f>
-        <v>1079</v>
+        <v>1301</v>
       </c>
     </row>
   </sheetData>
@@ -1802,8 +1907,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L28"/>
-  <sheetFormatPr defaultColWidth="8.66796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:L29"/>
+  <sheetFormatPr defaultColWidth="8.66796875" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="2" style="0" width="14"/>
@@ -1825,7 +1930,7 @@
       <c r="K1" s="10"/>
       <c r="L1" s="10"/>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
         <v>76</v>
       </c>
@@ -1863,825 +1968,879 @@
         <v>59</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="11" t="s">
+    <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="14" t="s">
         <v>77</v>
       </c>
-      <c r="B4" s="11" t="n">
+      <c r="B4" s="14" t="n">
+        <f aca="false">25+2</f>
+        <v>27</v>
+      </c>
+      <c r="C4" s="14" t="n">
+        <f aca="false">24+2</f>
+        <v>26</v>
+      </c>
+      <c r="D4" s="14" t="n">
+        <f aca="false">20+4</f>
+        <v>24</v>
+      </c>
+      <c r="E4" s="14" t="n">
+        <f aca="false">18+4</f>
+        <v>22</v>
+      </c>
+      <c r="F4" s="14" t="n">
+        <f aca="false">15+5</f>
+        <v>20</v>
+      </c>
+      <c r="G4" s="14" t="n">
+        <f aca="false">46+6</f>
+        <v>52</v>
+      </c>
+      <c r="H4" s="14" t="n">
+        <f aca="false">40+5</f>
+        <v>45</v>
+      </c>
+      <c r="I4" s="14"/>
+      <c r="J4" s="14" t="n">
+        <f aca="false">19+1</f>
+        <v>20</v>
+      </c>
+      <c r="K4" s="14" t="n">
+        <v>46</v>
+      </c>
+      <c r="L4" s="14" t="n">
+        <f aca="false">SUM(B4:K4)</f>
+        <v>282</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="14" t="s">
+        <v>78</v>
+      </c>
+      <c r="B5" s="14" t="n">
+        <v>19</v>
+      </c>
+      <c r="C5" s="14" t="n">
+        <v>20</v>
+      </c>
+      <c r="D5" s="14" t="n">
+        <v>7</v>
+      </c>
+      <c r="E5" s="14" t="n">
+        <v>19</v>
+      </c>
+      <c r="F5" s="14" t="n">
+        <v>34</v>
+      </c>
+      <c r="G5" s="14" t="n">
         <v>25</v>
       </c>
-      <c r="C4" s="11" t="n">
-        <v>24</v>
-      </c>
-      <c r="D4" s="11" t="n">
-        <v>20</v>
-      </c>
-      <c r="E4" s="11" t="n">
+      <c r="H5" s="14" t="n">
+        <v>21</v>
+      </c>
+      <c r="I5" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="J5" s="14" t="n">
+        <v>30</v>
+      </c>
+      <c r="K5" s="14" t="n">
         <v>18</v>
       </c>
-      <c r="F4" s="11" t="n">
-        <v>15</v>
-      </c>
-      <c r="G4" s="11" t="n">
-        <v>46</v>
-      </c>
-      <c r="H4" s="11" t="n">
-        <v>40</v>
-      </c>
-      <c r="I4" s="11"/>
-      <c r="J4" s="11" t="n">
-        <v>19</v>
-      </c>
-      <c r="K4" s="11" t="n">
-        <v>46</v>
-      </c>
-      <c r="L4" s="11" t="n">
-        <f aca="false">SUM(B4:K4)</f>
-        <v>253</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="11" t="s">
-        <v>78</v>
-      </c>
-      <c r="B5" s="11" t="n">
-        <v>19</v>
-      </c>
-      <c r="C5" s="11" t="n">
-        <v>20</v>
-      </c>
-      <c r="D5" s="11" t="n">
-        <v>7</v>
-      </c>
-      <c r="E5" s="11" t="n">
-        <v>19</v>
-      </c>
-      <c r="F5" s="11" t="n">
-        <v>34</v>
-      </c>
-      <c r="G5" s="11" t="n">
-        <v>25</v>
-      </c>
-      <c r="H5" s="11" t="n">
-        <v>21</v>
-      </c>
-      <c r="I5" s="11" t="n">
-        <v>6</v>
-      </c>
-      <c r="J5" s="11" t="n">
-        <v>30</v>
-      </c>
-      <c r="K5" s="11" t="n">
-        <v>18</v>
-      </c>
-      <c r="L5" s="11" t="n">
+      <c r="L5" s="14" t="n">
         <f aca="false">SUM(B5:K5)</f>
         <v>199</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="11" t="s">
+    <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="14" t="s">
         <v>79</v>
       </c>
-      <c r="B6" s="11" t="n">
+      <c r="B6" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="C6" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="D6" s="11" t="n">
+      <c r="C6" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="E6" s="11" t="n">
+      <c r="E6" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="F6" s="11" t="n">
+      <c r="F6" s="14" t="n">
         <v>17</v>
       </c>
-      <c r="G6" s="11" t="n">
+      <c r="G6" s="14" t="n">
         <v>26</v>
       </c>
-      <c r="H6" s="11" t="n">
+      <c r="H6" s="14" t="n">
         <v>20</v>
       </c>
-      <c r="I6" s="11" t="n">
+      <c r="I6" s="14" t="n">
         <v>9</v>
       </c>
-      <c r="J6" s="11" t="n">
+      <c r="J6" s="14" t="n">
         <v>28</v>
       </c>
-      <c r="K6" s="11" t="n">
+      <c r="K6" s="14" t="n">
         <v>28</v>
       </c>
-      <c r="L6" s="11" t="n">
+      <c r="L6" s="14" t="n">
         <f aca="false">SUM(B6:K6)</f>
         <v>142</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="11" t="s">
+    <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="14" t="s">
         <v>80</v>
       </c>
-      <c r="B7" s="11" t="n">
+      <c r="B7" s="14" t="n">
         <v>14</v>
       </c>
-      <c r="C7" s="11" t="n">
+      <c r="C7" s="14" t="n">
         <v>14</v>
       </c>
-      <c r="D7" s="11" t="n">
+      <c r="D7" s="14" t="n">
         <v>19</v>
       </c>
-      <c r="E7" s="11" t="n">
+      <c r="E7" s="14" t="n">
         <v>9</v>
       </c>
-      <c r="F7" s="11" t="n">
+      <c r="F7" s="14" t="n">
         <v>9</v>
       </c>
-      <c r="G7" s="11" t="n">
+      <c r="G7" s="14" t="n">
         <v>8</v>
       </c>
-      <c r="H7" s="11" t="n">
+      <c r="H7" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="I7" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="J7" s="11" t="n">
+      <c r="I7" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="J7" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="K7" s="11" t="n">
+      <c r="K7" s="14" t="n">
         <v>15</v>
       </c>
-      <c r="L7" s="11" t="n">
+      <c r="L7" s="14" t="n">
         <f aca="false">SUM(B7:K7)</f>
         <v>99</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="11" t="s">
+    <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="14" t="s">
         <v>81</v>
       </c>
-      <c r="B8" s="11" t="n">
+      <c r="B8" s="14" t="n">
         <v>10</v>
       </c>
-      <c r="C8" s="11" t="n">
+      <c r="C8" s="14" t="n">
         <v>10</v>
       </c>
-      <c r="D8" s="11" t="n">
+      <c r="D8" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="E8" s="11" t="n">
+      <c r="E8" s="14" t="n">
         <v>10</v>
       </c>
-      <c r="F8" s="11" t="n">
+      <c r="F8" s="14" t="n">
         <v>6</v>
       </c>
-      <c r="G8" s="11" t="n">
+      <c r="G8" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="H8" s="11" t="n">
+      <c r="H8" s="14" t="n">
         <v>10</v>
       </c>
-      <c r="I8" s="11" t="n">
+      <c r="I8" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="J8" s="11" t="n">
+      <c r="J8" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="K8" s="11" t="n">
+      <c r="K8" s="14" t="n">
         <v>8</v>
       </c>
-      <c r="L8" s="11" t="n">
+      <c r="L8" s="14" t="n">
         <f aca="false">SUM(B8:K8)</f>
         <v>71</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="11" t="s">
+    <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="14" t="s">
         <v>82</v>
       </c>
-      <c r="B9" s="11" t="n">
+      <c r="B9" s="14" t="n">
         <v>7</v>
       </c>
-      <c r="C9" s="11" t="n">
+      <c r="C9" s="14" t="n">
         <v>7</v>
       </c>
-      <c r="D9" s="11" t="n">
+      <c r="D9" s="14" t="n">
         <v>16</v>
       </c>
-      <c r="E9" s="11" t="n">
+      <c r="E9" s="14" t="n">
         <v>13</v>
       </c>
-      <c r="F9" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="G9" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="H9" s="11" t="n">
+      <c r="F9" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="G9" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="H9" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="I9" s="11"/>
-      <c r="J9" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="K9" s="11" t="n">
+      <c r="I9" s="14"/>
+      <c r="J9" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="K9" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="L9" s="11" t="n">
+      <c r="L9" s="14" t="n">
         <f aca="false">SUM(B9:K9)</f>
         <v>57</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="11" t="s">
+    <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="14" t="s">
         <v>83</v>
       </c>
-      <c r="B10" s="11" t="n">
+      <c r="B10" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="C10" s="11" t="n">
+      <c r="C10" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="D10" s="11" t="n">
+      <c r="D10" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="E10" s="11" t="n">
+      <c r="E10" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="F10" s="11" t="n">
+      <c r="F10" s="14" t="n">
         <v>7</v>
       </c>
-      <c r="G10" s="11" t="n">
+      <c r="G10" s="14" t="n">
         <v>6</v>
       </c>
-      <c r="H10" s="11" t="n">
+      <c r="H10" s="14" t="n">
         <v>6</v>
       </c>
-      <c r="I10" s="11" t="n">
+      <c r="I10" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="J10" s="11" t="n">
+      <c r="J10" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="K10" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="L10" s="11" t="n">
+      <c r="K10" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="L10" s="14" t="n">
         <f aca="false">SUM(B10:K10)</f>
         <v>44</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="11" t="s">
+    <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="14" t="s">
         <v>84</v>
       </c>
-      <c r="B11" s="11" t="n">
+      <c r="B11" s="14" t="n">
         <v>12</v>
       </c>
-      <c r="C11" s="11" t="n">
+      <c r="C11" s="14" t="n">
         <v>8</v>
       </c>
-      <c r="D11" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="E11" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="F11" s="11" t="n">
+      <c r="D11" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="E11" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="F11" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="G11" s="11" t="n">
+      <c r="G11" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="H11" s="11" t="n">
+      <c r="H11" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="I11" s="11"/>
-      <c r="J11" s="11" t="n">
+      <c r="I11" s="14"/>
+      <c r="J11" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="K11" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="L11" s="11" t="n">
+      <c r="K11" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="L11" s="14" t="n">
         <f aca="false">SUM(B11:K11)</f>
         <v>39</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="11" t="s">
+    <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="14" t="s">
         <v>85</v>
       </c>
-      <c r="B12" s="11" t="n">
+      <c r="B12" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="C12" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="D12" s="11" t="n">
+      <c r="C12" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="D12" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="E12" s="11" t="n">
+      <c r="E12" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="F12" s="11" t="n">
+      <c r="F12" s="14" t="n">
         <v>7</v>
       </c>
-      <c r="G12" s="11" t="n">
+      <c r="G12" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="H12" s="11" t="n">
+      <c r="H12" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="I12" s="11" t="n">
+      <c r="I12" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="J12" s="11" t="n">
+      <c r="J12" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="K12" s="11"/>
-      <c r="L12" s="11" t="n">
+      <c r="K12" s="14"/>
+      <c r="L12" s="14" t="n">
         <f aca="false">SUM(B12:K12)</f>
         <v>36</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="11" t="s">
+    <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="14" t="s">
         <v>86</v>
       </c>
-      <c r="B13" s="11"/>
-      <c r="C13" s="11" t="n">
+      <c r="B13" s="14"/>
+      <c r="C13" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="D13" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="E13" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="F13" s="11" t="n">
+      <c r="D13" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="F13" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="G13" s="11" t="n">
+      <c r="G13" s="14" t="n">
         <v>7</v>
       </c>
-      <c r="H13" s="11" t="n">
+      <c r="H13" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="I13" s="11"/>
-      <c r="J13" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="K13" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="L13" s="11" t="n">
+      <c r="I13" s="14"/>
+      <c r="J13" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="K13" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="L13" s="14" t="n">
         <f aca="false">SUM(B13:K13)</f>
         <v>22</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="11" t="s">
+    <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="14" t="s">
         <v>87</v>
       </c>
-      <c r="B14" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="C14" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="D14" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="E14" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="F14" s="11"/>
-      <c r="G14" s="11" t="n">
+      <c r="B14" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="C14" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="F14" s="14"/>
+      <c r="G14" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="H14" s="11" t="n">
+      <c r="H14" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="I14" s="11"/>
-      <c r="J14" s="11" t="n">
+      <c r="I14" s="14"/>
+      <c r="J14" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="K14" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="L14" s="11" t="n">
+      <c r="K14" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="L14" s="14" t="n">
         <f aca="false">SUM(B14:K14)</f>
         <v>19</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="11" t="s">
+    <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="14" t="s">
         <v>88</v>
       </c>
-      <c r="B15" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="C15" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="D15" s="11"/>
-      <c r="E15" s="11" t="n">
+      <c r="B15" s="14" t="n">
+        <f aca="false">1+2</f>
         <v>3</v>
       </c>
-      <c r="F15" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="G15" s="11" t="n">
-        <v>5</v>
-      </c>
-      <c r="H15" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="I15" s="11"/>
-      <c r="J15" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="K15" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="L15" s="11" t="n">
+      <c r="C15" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="D15" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="E15" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="F15" s="14" t="n">
+        <f aca="false">1+1</f>
+        <v>2</v>
+      </c>
+      <c r="G15" s="14" t="n">
+        <f aca="false">5+2</f>
+        <v>7</v>
+      </c>
+      <c r="H15" s="14" t="n">
+        <f aca="false">1+3</f>
+        <v>4</v>
+      </c>
+      <c r="I15" s="14"/>
+      <c r="J15" s="14" t="n">
+        <f aca="false">1+1</f>
+        <v>2</v>
+      </c>
+      <c r="K15" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="L15" s="14" t="n">
         <f aca="false">SUM(B15:K15)</f>
-        <v>16</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="11" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="14" t="s">
         <v>89</v>
       </c>
-      <c r="B16" s="11" t="n">
+      <c r="B16" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="C16" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="D16" s="11" t="n">
+      <c r="C16" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="D16" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="E16" s="11"/>
-      <c r="F16" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="G16" s="11"/>
-      <c r="H16" s="11" t="n">
+      <c r="E16" s="14"/>
+      <c r="F16" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="G16" s="14"/>
+      <c r="H16" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="I16" s="11"/>
-      <c r="J16" s="11" t="n">
+      <c r="I16" s="14"/>
+      <c r="J16" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="K16" s="11"/>
-      <c r="L16" s="11" t="n">
+      <c r="K16" s="14"/>
+      <c r="L16" s="14" t="n">
         <f aca="false">SUM(B16:K16)</f>
         <v>16</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="11" t="s">
+    <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="14" t="s">
         <v>90</v>
       </c>
-      <c r="B17" s="11"/>
-      <c r="C17" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="D17" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="E17" s="11"/>
-      <c r="F17" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="G17" s="11"/>
-      <c r="H17" s="11" t="n">
+      <c r="B17" s="14"/>
+      <c r="C17" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="D17" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="E17" s="14"/>
+      <c r="F17" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="G17" s="14"/>
+      <c r="H17" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="I17" s="11"/>
-      <c r="J17" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="K17" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="L17" s="11" t="n">
+      <c r="I17" s="14"/>
+      <c r="J17" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="K17" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="L17" s="14" t="n">
         <f aca="false">SUM(B17:K17)</f>
         <v>11</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="11" t="s">
+    <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="14" t="s">
         <v>91</v>
       </c>
-      <c r="B18" s="11"/>
-      <c r="C18" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="D18" s="11"/>
-      <c r="E18" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="F18" s="11" t="n">
+      <c r="B18" s="14"/>
+      <c r="C18" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="D18" s="14"/>
+      <c r="E18" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="F18" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="G18" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="H18" s="11"/>
-      <c r="I18" s="11"/>
-      <c r="J18" s="11"/>
-      <c r="K18" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="L18" s="11" t="n">
+      <c r="G18" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="H18" s="14"/>
+      <c r="I18" s="14"/>
+      <c r="J18" s="14"/>
+      <c r="K18" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="L18" s="14" t="n">
         <f aca="false">SUM(B18:K18)</f>
         <v>10</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="11" t="s">
+    <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="14" t="s">
         <v>92</v>
       </c>
-      <c r="B19" s="11" t="n">
+      <c r="B19" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="C19" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="D19" s="11"/>
-      <c r="E19" s="11"/>
-      <c r="F19" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="G19" s="11"/>
-      <c r="H19" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="I19" s="11"/>
-      <c r="J19" s="11"/>
-      <c r="K19" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="L19" s="11" t="n">
+      <c r="C19" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="D19" s="14"/>
+      <c r="E19" s="14"/>
+      <c r="F19" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="G19" s="14"/>
+      <c r="H19" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="I19" s="14"/>
+      <c r="J19" s="14"/>
+      <c r="K19" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="L19" s="14" t="n">
         <f aca="false">SUM(B19:K19)</f>
         <v>10</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="11" t="s">
+    <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="14" t="s">
         <v>93</v>
       </c>
-      <c r="B20" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="C20" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="D20" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="E20" s="11"/>
-      <c r="F20" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="G20" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="H20" s="11"/>
-      <c r="I20" s="11"/>
-      <c r="J20" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="K20" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="L20" s="11" t="n">
+      <c r="B20" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="C20" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="D20" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="E20" s="14"/>
+      <c r="F20" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="G20" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="H20" s="14"/>
+      <c r="I20" s="14"/>
+      <c r="J20" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="K20" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="L20" s="14" t="n">
         <f aca="false">SUM(B20:K20)</f>
         <v>8</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="11" t="s">
+    <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="14" t="s">
         <v>94</v>
       </c>
-      <c r="B21" s="11"/>
-      <c r="C21" s="11"/>
-      <c r="D21" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="E21" s="11"/>
-      <c r="F21" s="11"/>
-      <c r="G21" s="11" t="n">
+      <c r="B21" s="14"/>
+      <c r="C21" s="14"/>
+      <c r="D21" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="E21" s="14"/>
+      <c r="F21" s="14"/>
+      <c r="G21" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="H21" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="I21" s="11"/>
-      <c r="J21" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="K21" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="L21" s="11" t="n">
+      <c r="H21" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="I21" s="14"/>
+      <c r="J21" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="K21" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="L21" s="14" t="n">
         <f aca="false">SUM(B21:K21)</f>
         <v>7</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="11" t="s">
+    <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="14" t="s">
         <v>95</v>
       </c>
-      <c r="B22" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="C22" s="11"/>
-      <c r="D22" s="11"/>
-      <c r="E22" s="11"/>
-      <c r="F22" s="11"/>
-      <c r="G22" s="11"/>
-      <c r="H22" s="11" t="n">
+      <c r="B22" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="C22" s="14"/>
+      <c r="D22" s="14"/>
+      <c r="E22" s="14"/>
+      <c r="F22" s="14"/>
+      <c r="G22" s="14"/>
+      <c r="H22" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="I22" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="J22" s="11"/>
-      <c r="K22" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="L22" s="11" t="n">
+      <c r="I22" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="J22" s="14"/>
+      <c r="K22" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="L22" s="14" t="n">
         <f aca="false">SUM(B22:K22)</f>
         <v>6</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="11" t="s">
+    <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="14" t="s">
         <v>96</v>
       </c>
-      <c r="B23" s="11"/>
-      <c r="C23" s="11"/>
-      <c r="D23" s="11"/>
-      <c r="E23" s="11"/>
-      <c r="F23" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="G23" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="H23" s="11"/>
-      <c r="I23" s="11"/>
-      <c r="J23" s="11"/>
-      <c r="K23" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="L23" s="11" t="n">
+      <c r="B23" s="14"/>
+      <c r="C23" s="14"/>
+      <c r="D23" s="14"/>
+      <c r="E23" s="14"/>
+      <c r="F23" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="G23" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="H23" s="14"/>
+      <c r="I23" s="14"/>
+      <c r="J23" s="14"/>
+      <c r="K23" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="L23" s="14" t="n">
         <f aca="false">SUM(B23:K23)</f>
         <v>4</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="11" t="s">
+    <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="14" t="s">
         <v>97</v>
       </c>
-      <c r="B24" s="11"/>
-      <c r="C24" s="11"/>
-      <c r="D24" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="E24" s="11"/>
-      <c r="F24" s="11"/>
-      <c r="G24" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="H24" s="11"/>
-      <c r="I24" s="11"/>
-      <c r="J24" s="11"/>
-      <c r="K24" s="11"/>
-      <c r="L24" s="11" t="n">
+      <c r="B24" s="14"/>
+      <c r="C24" s="14"/>
+      <c r="D24" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="E24" s="14"/>
+      <c r="F24" s="14"/>
+      <c r="G24" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="H24" s="14"/>
+      <c r="I24" s="14"/>
+      <c r="J24" s="14"/>
+      <c r="K24" s="14"/>
+      <c r="L24" s="14" t="n">
         <f aca="false">SUM(B24:K24)</f>
         <v>3</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="11" t="s">
+    <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="14" t="s">
         <v>98</v>
       </c>
-      <c r="B25" s="11"/>
-      <c r="C25" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="D25" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="E25" s="11"/>
-      <c r="F25" s="11"/>
-      <c r="G25" s="11"/>
-      <c r="H25" s="11"/>
-      <c r="I25" s="11"/>
-      <c r="J25" s="11"/>
-      <c r="K25" s="11"/>
-      <c r="L25" s="11" t="n">
+      <c r="B25" s="14"/>
+      <c r="C25" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="D25" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="E25" s="14"/>
+      <c r="F25" s="14"/>
+      <c r="G25" s="14"/>
+      <c r="H25" s="14"/>
+      <c r="I25" s="14"/>
+      <c r="J25" s="14"/>
+      <c r="K25" s="14"/>
+      <c r="L25" s="14" t="n">
         <f aca="false">SUM(B25:K25)</f>
         <v>3</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="11" t="s">
+    <row r="26" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="14" t="s">
         <v>99</v>
       </c>
-      <c r="B26" s="11"/>
-      <c r="C26" s="11"/>
-      <c r="D26" s="11"/>
-      <c r="E26" s="11"/>
-      <c r="F26" s="11"/>
-      <c r="G26" s="11"/>
-      <c r="H26" s="11"/>
-      <c r="I26" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="J26" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="K26" s="11"/>
-      <c r="L26" s="11" t="n">
+      <c r="B26" s="14"/>
+      <c r="C26" s="14"/>
+      <c r="D26" s="14"/>
+      <c r="E26" s="14"/>
+      <c r="F26" s="14"/>
+      <c r="G26" s="14"/>
+      <c r="H26" s="14"/>
+      <c r="I26" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="J26" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="K26" s="14"/>
+      <c r="L26" s="14" t="n">
         <f aca="false">SUM(B26:K26)</f>
         <v>2</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="11" t="s">
+    <row r="27" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="14" t="s">
         <v>100</v>
       </c>
-      <c r="B27" s="11"/>
-      <c r="C27" s="11"/>
-      <c r="D27" s="11"/>
-      <c r="E27" s="11"/>
-      <c r="F27" s="11"/>
-      <c r="G27" s="11"/>
-      <c r="H27" s="11"/>
-      <c r="I27" s="11"/>
-      <c r="J27" s="11"/>
-      <c r="K27" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="L27" s="11" t="n">
+      <c r="B27" s="14"/>
+      <c r="C27" s="14"/>
+      <c r="D27" s="14"/>
+      <c r="E27" s="14"/>
+      <c r="F27" s="14"/>
+      <c r="G27" s="14"/>
+      <c r="H27" s="14"/>
+      <c r="I27" s="14"/>
+      <c r="J27" s="14"/>
+      <c r="K27" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="L27" s="14" t="n">
         <f aca="false">SUM(B27:K27)</f>
         <v>1</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="7" t="s">
+    <row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="14" t="s">
+        <v>101</v>
+      </c>
+      <c r="B28" s="14" t="n">
+        <v>14</v>
+      </c>
+      <c r="C28" s="14" t="n">
+        <v>27</v>
+      </c>
+      <c r="D28" s="14" t="n">
+        <v>27</v>
+      </c>
+      <c r="E28" s="14" t="n">
+        <v>26</v>
+      </c>
+      <c r="F28" s="14" t="n">
+        <v>22</v>
+      </c>
+      <c r="G28" s="14" t="n">
+        <v>27</v>
+      </c>
+      <c r="H28" s="14" t="n">
+        <v>27</v>
+      </c>
+      <c r="I28" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="J28" s="14" t="n">
+        <v>33</v>
+      </c>
+      <c r="K28" s="14" t="n">
+        <v>16</v>
+      </c>
+      <c r="L28" s="14" t="n">
+        <f aca="false">SUM(B28:K28)</f>
+        <v>219</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="7" t="s">
         <v>74</v>
       </c>
-      <c r="B28" s="7" t="n">
-        <f aca="false">SUM(B4:B27)</f>
-        <v>111</v>
-      </c>
-      <c r="C28" s="7" t="n">
-        <f aca="false">SUM(C4:C27)</f>
-        <v>107</v>
-      </c>
-      <c r="D28" s="7" t="n">
-        <f aca="false">SUM(D4:D27)</f>
-        <v>91</v>
-      </c>
-      <c r="E28" s="7" t="n">
-        <f aca="false">SUM(E4:E27)</f>
-        <v>88</v>
-      </c>
-      <c r="F28" s="7" t="n">
-        <f aca="false">SUM(F4:F27)</f>
-        <v>114</v>
-      </c>
-      <c r="G28" s="7" t="n">
-        <f aca="false">SUM(G4:G27)</f>
-        <v>150</v>
-      </c>
-      <c r="H28" s="7" t="n">
-        <f aca="false">SUM(H4:H27)</f>
+      <c r="B29" s="7" t="n">
+        <f aca="false">SUM(B4:B28)</f>
+        <v>129</v>
+      </c>
+      <c r="C29" s="7" t="n">
+        <f aca="false">SUM(C4:C28)</f>
         <v>136</v>
       </c>
-      <c r="I28" s="7" t="n">
-        <f aca="false">SUM(I4:I27)</f>
+      <c r="D29" s="7" t="n">
+        <f aca="false">SUM(D4:D28)</f>
+        <v>124</v>
+      </c>
+      <c r="E29" s="7" t="n">
+        <f aca="false">SUM(E4:E28)</f>
+        <v>118</v>
+      </c>
+      <c r="F29" s="7" t="n">
+        <f aca="false">SUM(F4:F28)</f>
+        <v>142</v>
+      </c>
+      <c r="G29" s="7" t="n">
+        <f aca="false">SUM(G4:G28)</f>
+        <v>185</v>
+      </c>
+      <c r="H29" s="7" t="n">
+        <f aca="false">SUM(H4:H28)</f>
+        <v>171</v>
+      </c>
+      <c r="I29" s="7" t="n">
+        <f aca="false">SUM(I4:I28)</f>
         <v>30</v>
       </c>
-      <c r="J28" s="7" t="n">
-        <f aca="false">SUM(J4:J27)</f>
-        <v>112</v>
-      </c>
-      <c r="K28" s="7" t="n">
-        <f aca="false">SUM(K4:K27)</f>
-        <v>139</v>
-      </c>
-      <c r="L28" s="7" t="n">
-        <f aca="false">SUM(L4:L27)</f>
-        <v>1078</v>
+      <c r="J29" s="7" t="n">
+        <f aca="false">SUM(J4:J28)</f>
+        <v>147</v>
+      </c>
+      <c r="K29" s="7" t="n">
+        <f aca="false">SUM(K4:K28)</f>
+        <v>155</v>
+      </c>
+      <c r="L29" s="7" t="n">
+        <f aca="false">SUM(L4:L28)</f>
+        <v>1337</v>
       </c>
     </row>
   </sheetData>
@@ -2703,8 +2862,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L28"/>
-  <sheetFormatPr defaultColWidth="8.66796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:L29"/>
+  <sheetFormatPr defaultColWidth="8.66796875" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="2" style="0" width="14"/>
@@ -2712,7 +2871,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="10" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B1" s="10"/>
       <c r="C1" s="10"/>
@@ -2726,7 +2885,7 @@
       <c r="K1" s="10"/>
       <c r="L1" s="10"/>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
         <v>76</v>
       </c>
@@ -2764,837 +2923,890 @@
         <v>59</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="11" t="s">
+    <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="14" t="s">
         <v>89</v>
       </c>
-      <c r="B4" s="11" t="n">
-        <v>179</v>
-      </c>
-      <c r="C4" s="11" t="n">
-        <v>283.5</v>
-      </c>
-      <c r="D4" s="11" t="n">
-        <v>132.75</v>
-      </c>
-      <c r="E4" s="11" t="n">
-        <v>160</v>
-      </c>
-      <c r="F4" s="11" t="n">
-        <v>195</v>
-      </c>
-      <c r="G4" s="11" t="n">
-        <v>224.75</v>
-      </c>
-      <c r="H4" s="11" t="n">
-        <v>202.65</v>
-      </c>
-      <c r="I4" s="11" t="n">
+      <c r="B4" s="14" t="n">
+        <f aca="false">179+21</f>
+        <v>200</v>
+      </c>
+      <c r="C4" s="14" t="n">
+        <f aca="false">283.5+4</f>
+        <v>287.5</v>
+      </c>
+      <c r="D4" s="14" t="n">
+        <f aca="false">132.75+33</f>
+        <v>165.75</v>
+      </c>
+      <c r="E4" s="14" t="n">
+        <f aca="false">160+13</f>
+        <v>173</v>
+      </c>
+      <c r="F4" s="14" t="n">
+        <f aca="false">195+47</f>
+        <v>242</v>
+      </c>
+      <c r="G4" s="14" t="n">
+        <f aca="false">224.75+19</f>
+        <v>243.75</v>
+      </c>
+      <c r="H4" s="14" t="n">
+        <f aca="false">202.65+23</f>
+        <v>225.65</v>
+      </c>
+      <c r="I4" s="14" t="n">
         <v>276.75</v>
       </c>
-      <c r="J4" s="11" t="n">
-        <v>298.25</v>
-      </c>
-      <c r="K4" s="11" t="n">
+      <c r="J4" s="14" t="n">
+        <f aca="false">298.25+1</f>
+        <v>299.25</v>
+      </c>
+      <c r="K4" s="14" t="n">
         <v>59.25</v>
       </c>
-      <c r="L4" s="11" t="n">
+      <c r="L4" s="14" t="n">
         <f aca="false">SUM(B4:K4)</f>
-        <v>2011.9</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="11" t="s">
+        <v>2172.9</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="14" t="s">
         <v>79</v>
       </c>
-      <c r="B5" s="11" t="n">
+      <c r="B5" s="14" t="n">
         <v>13</v>
       </c>
-      <c r="C5" s="11" t="n">
+      <c r="C5" s="14" t="n">
         <v>6</v>
       </c>
-      <c r="D5" s="11" t="n">
+      <c r="D5" s="14" t="n">
         <v>34.5</v>
       </c>
-      <c r="E5" s="11" t="n">
+      <c r="E5" s="14" t="n">
         <v>36</v>
       </c>
-      <c r="F5" s="11" t="n">
+      <c r="F5" s="14" t="n">
         <v>82</v>
       </c>
-      <c r="G5" s="11" t="n">
+      <c r="G5" s="14" t="n">
         <v>129.75</v>
       </c>
-      <c r="H5" s="11" t="n">
+      <c r="H5" s="14" t="n">
         <v>94.5</v>
       </c>
-      <c r="I5" s="11" t="n">
+      <c r="I5" s="14" t="n">
         <v>74.5</v>
       </c>
-      <c r="J5" s="11" t="n">
+      <c r="J5" s="14" t="n">
         <v>137</v>
       </c>
-      <c r="K5" s="11" t="n">
+      <c r="K5" s="14" t="n">
         <v>119.5</v>
       </c>
-      <c r="L5" s="11" t="n">
+      <c r="L5" s="14" t="n">
         <f aca="false">SUM(B5:K5)</f>
         <v>726.75</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="11" t="s">
+    <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="B6" s="11" t="n">
+      <c r="B6" s="14" t="n">
         <v>149.75</v>
       </c>
-      <c r="C6" s="11" t="n">
+      <c r="C6" s="14" t="n">
         <v>25.5</v>
       </c>
-      <c r="D6" s="11" t="n">
+      <c r="D6" s="14" t="n">
         <v>53.25</v>
       </c>
-      <c r="E6" s="11" t="n">
+      <c r="E6" s="14" t="n">
         <v>60.8</v>
       </c>
-      <c r="F6" s="11" t="n">
+      <c r="F6" s="14" t="n">
         <v>96.25</v>
       </c>
-      <c r="G6" s="11" t="n">
+      <c r="G6" s="14" t="n">
         <v>99</v>
       </c>
-      <c r="H6" s="11" t="n">
+      <c r="H6" s="14" t="n">
         <v>71.65</v>
       </c>
-      <c r="I6" s="11" t="n">
+      <c r="I6" s="14" t="n">
         <v>17.25</v>
       </c>
-      <c r="J6" s="11" t="n">
+      <c r="J6" s="14" t="n">
         <v>96.75</v>
       </c>
-      <c r="K6" s="11" t="n">
+      <c r="K6" s="14" t="n">
         <v>29.25</v>
       </c>
-      <c r="L6" s="11" t="n">
+      <c r="L6" s="14" t="n">
         <f aca="false">SUM(B6:K6)</f>
         <v>699.45</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="11" t="s">
+    <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="14" t="s">
         <v>77</v>
       </c>
-      <c r="B7" s="11" t="n">
+      <c r="B7" s="14" t="n">
         <v>27.5</v>
       </c>
-      <c r="C7" s="11" t="n">
+      <c r="C7" s="14" t="n">
         <v>62.25</v>
       </c>
-      <c r="D7" s="11" t="n">
+      <c r="D7" s="14" t="n">
         <v>102.5</v>
       </c>
-      <c r="E7" s="11" t="n">
+      <c r="E7" s="14" t="n">
         <v>60</v>
       </c>
-      <c r="F7" s="11" t="n">
+      <c r="F7" s="14" t="n">
         <v>26.75</v>
       </c>
-      <c r="G7" s="11" t="n">
+      <c r="G7" s="14" t="n">
         <v>70.55</v>
       </c>
-      <c r="H7" s="11" t="n">
+      <c r="H7" s="14" t="n">
         <v>84.85</v>
       </c>
-      <c r="I7" s="11" t="n">
+      <c r="I7" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="J7" s="11" t="n">
+      <c r="J7" s="14" t="n">
         <v>39.75</v>
       </c>
-      <c r="K7" s="11" t="n">
+      <c r="K7" s="14" t="n">
         <v>95.5</v>
       </c>
-      <c r="L7" s="11" t="n">
+      <c r="L7" s="14" t="n">
         <f aca="false">SUM(B7:K7)</f>
         <v>572.65</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="11" t="s">
+    <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="14" t="s">
         <v>81</v>
       </c>
-      <c r="B8" s="11" t="n">
+      <c r="B8" s="14" t="n">
         <v>89</v>
       </c>
-      <c r="C8" s="11" t="n">
+      <c r="C8" s="14" t="n">
         <v>65.5</v>
       </c>
-      <c r="D8" s="11" t="n">
+      <c r="D8" s="14" t="n">
         <v>28</v>
       </c>
-      <c r="E8" s="11" t="n">
+      <c r="E8" s="14" t="n">
         <v>66</v>
       </c>
-      <c r="F8" s="11" t="n">
+      <c r="F8" s="14" t="n">
         <v>19.75</v>
       </c>
-      <c r="G8" s="11" t="n">
+      <c r="G8" s="14" t="n">
         <v>9.75</v>
       </c>
-      <c r="H8" s="11" t="n">
+      <c r="H8" s="14" t="n">
         <v>32.25</v>
       </c>
-      <c r="I8" s="11" t="n">
+      <c r="I8" s="14" t="n">
         <v>11.5</v>
       </c>
-      <c r="J8" s="11" t="n">
+      <c r="J8" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="K8" s="11" t="n">
+      <c r="K8" s="14" t="n">
         <v>23.5</v>
       </c>
-      <c r="L8" s="11" t="n">
+      <c r="L8" s="14" t="n">
         <f aca="false">SUM(B8:K8)</f>
         <v>350.25</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="11" t="s">
+    <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="14" t="s">
         <v>82</v>
       </c>
-      <c r="B9" s="11" t="n">
+      <c r="B9" s="14" t="n">
         <v>29.25</v>
       </c>
-      <c r="C9" s="11" t="n">
+      <c r="C9" s="14" t="n">
         <v>43.5</v>
       </c>
-      <c r="D9" s="11" t="n">
+      <c r="D9" s="14" t="n">
         <v>71.5</v>
       </c>
-      <c r="E9" s="11" t="n">
+      <c r="E9" s="14" t="n">
         <v>84</v>
       </c>
-      <c r="F9" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="G9" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="H9" s="11" t="n">
+      <c r="F9" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="G9" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="H9" s="14" t="n">
         <v>34</v>
       </c>
-      <c r="I9" s="11"/>
-      <c r="J9" s="11" t="n">
+      <c r="I9" s="14"/>
+      <c r="J9" s="14" t="n">
         <v>21.25</v>
       </c>
-      <c r="K9" s="11" t="n">
+      <c r="K9" s="14" t="n">
         <v>12</v>
       </c>
-      <c r="L9" s="11" t="n">
+      <c r="L9" s="14" t="n">
         <f aca="false">SUM(B9:K9)</f>
         <v>297.5</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="11" t="s">
+    <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="14" t="s">
         <v>83</v>
       </c>
-      <c r="B10" s="11" t="n">
+      <c r="B10" s="14" t="n">
         <v>16.75</v>
       </c>
-      <c r="C10" s="11" t="n">
+      <c r="C10" s="14" t="n">
         <v>8</v>
       </c>
-      <c r="D10" s="11" t="n">
+      <c r="D10" s="14" t="n">
         <v>38</v>
       </c>
-      <c r="E10" s="11" t="n">
+      <c r="E10" s="14" t="n">
         <v>40.5</v>
       </c>
-      <c r="F10" s="11" t="n">
+      <c r="F10" s="14" t="n">
         <v>37.5</v>
       </c>
-      <c r="G10" s="11" t="n">
+      <c r="G10" s="14" t="n">
         <v>32</v>
       </c>
-      <c r="H10" s="11" t="n">
+      <c r="H10" s="14" t="n">
         <v>34.5</v>
       </c>
-      <c r="I10" s="11" t="n">
+      <c r="I10" s="14" t="n">
         <v>6.5</v>
       </c>
-      <c r="J10" s="11" t="n">
+      <c r="J10" s="14" t="n">
         <v>29</v>
       </c>
-      <c r="K10" s="11" t="n">
+      <c r="K10" s="14" t="n">
         <v>2.5</v>
       </c>
-      <c r="L10" s="11" t="n">
+      <c r="L10" s="14" t="n">
         <f aca="false">SUM(B10:K10)</f>
         <v>245.25</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="11" t="s">
+    <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="14" t="s">
         <v>84</v>
       </c>
-      <c r="B11" s="11" t="n">
+      <c r="B11" s="14" t="n">
         <v>74</v>
       </c>
-      <c r="C11" s="11" t="n">
+      <c r="C11" s="14" t="n">
         <v>53.5</v>
       </c>
-      <c r="D11" s="11" t="n">
+      <c r="D11" s="14" t="n">
         <v>28.5</v>
       </c>
-      <c r="E11" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="F11" s="11" t="n">
+      <c r="E11" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="F11" s="14" t="n">
         <v>24.75</v>
       </c>
-      <c r="G11" s="11" t="n">
+      <c r="G11" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="H11" s="11" t="n">
+      <c r="H11" s="14" t="n">
         <v>21.5</v>
       </c>
-      <c r="I11" s="11"/>
-      <c r="J11" s="11" t="n">
+      <c r="I11" s="14"/>
+      <c r="J11" s="14" t="n">
         <v>21</v>
       </c>
-      <c r="K11" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="L11" s="11" t="n">
+      <c r="K11" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="L11" s="14" t="n">
         <f aca="false">SUM(B11:K11)</f>
         <v>230.25</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="11" t="s">
+    <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="14" t="s">
         <v>85</v>
       </c>
-      <c r="B12" s="11" t="n">
+      <c r="B12" s="14" t="n">
         <v>24.25</v>
       </c>
-      <c r="C12" s="11" t="n">
+      <c r="C12" s="14" t="n">
         <v>15</v>
       </c>
-      <c r="D12" s="11" t="n">
+      <c r="D12" s="14" t="n">
         <v>11.5</v>
       </c>
-      <c r="E12" s="11" t="n">
+      <c r="E12" s="14" t="n">
         <v>20.5</v>
       </c>
-      <c r="F12" s="11" t="n">
+      <c r="F12" s="14" t="n">
         <v>32.5</v>
       </c>
-      <c r="G12" s="11" t="n">
+      <c r="G12" s="14" t="n">
         <v>11</v>
       </c>
-      <c r="H12" s="11" t="n">
+      <c r="H12" s="14" t="n">
         <v>31</v>
       </c>
-      <c r="I12" s="11" t="n">
+      <c r="I12" s="14" t="n">
         <v>29.25</v>
       </c>
-      <c r="J12" s="11" t="n">
+      <c r="J12" s="14" t="n">
         <v>33.25</v>
       </c>
-      <c r="K12" s="11"/>
-      <c r="L12" s="11" t="n">
+      <c r="K12" s="14"/>
+      <c r="L12" s="14" t="n">
         <f aca="false">SUM(B12:K12)</f>
         <v>208.25</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="11" t="s">
+    <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="14" t="s">
         <v>80</v>
       </c>
-      <c r="B13" s="11" t="n">
+      <c r="B13" s="14" t="n">
         <v>9</v>
       </c>
-      <c r="C13" s="11" t="n">
+      <c r="C13" s="14" t="n">
         <v>13</v>
       </c>
-      <c r="D13" s="11" t="n">
+      <c r="D13" s="14" t="n">
         <v>18.25</v>
       </c>
-      <c r="E13" s="11" t="n">
+      <c r="E13" s="14" t="n">
         <v>17.5</v>
       </c>
-      <c r="F13" s="11" t="n">
+      <c r="F13" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="G13" s="11" t="n">
+      <c r="G13" s="14" t="n">
         <v>7.75</v>
       </c>
-      <c r="H13" s="11" t="n">
+      <c r="H13" s="14" t="n">
         <v>5.25</v>
       </c>
-      <c r="I13" s="11" t="n">
+      <c r="I13" s="14" t="n">
         <v>2.5</v>
       </c>
-      <c r="J13" s="11" t="n">
+      <c r="J13" s="14" t="n">
         <v>4.75</v>
       </c>
-      <c r="K13" s="11" t="n">
+      <c r="K13" s="14" t="n">
         <v>8.5</v>
       </c>
-      <c r="L13" s="11" t="n">
+      <c r="L13" s="14" t="n">
         <f aca="false">SUM(B13:K13)</f>
         <v>91.5</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="11" t="s">
+    <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="14" t="s">
         <v>91</v>
       </c>
-      <c r="B14" s="11"/>
-      <c r="C14" s="11" t="n">
+      <c r="B14" s="14"/>
+      <c r="C14" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="D14" s="11"/>
-      <c r="E14" s="11" t="n">
+      <c r="D14" s="14"/>
+      <c r="E14" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="F14" s="11" t="n">
+      <c r="F14" s="14" t="n">
         <v>48</v>
       </c>
-      <c r="G14" s="11" t="n">
+      <c r="G14" s="14" t="n">
         <v>10.5</v>
       </c>
-      <c r="H14" s="11"/>
-      <c r="I14" s="11"/>
-      <c r="J14" s="11"/>
-      <c r="K14" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="L14" s="11" t="n">
+      <c r="H14" s="14"/>
+      <c r="I14" s="14"/>
+      <c r="J14" s="14"/>
+      <c r="K14" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="L14" s="14" t="n">
         <f aca="false">SUM(B14:K14)</f>
         <v>68.5</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="11" t="s">
+    <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="14" t="s">
         <v>86</v>
       </c>
-      <c r="B15" s="11"/>
-      <c r="C15" s="11" t="n">
+      <c r="B15" s="14"/>
+      <c r="C15" s="14" t="n">
         <v>14.5</v>
       </c>
-      <c r="D15" s="11" t="n">
+      <c r="D15" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="E15" s="11" t="n">
+      <c r="E15" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="F15" s="11" t="n">
+      <c r="F15" s="14" t="n">
         <v>3.25</v>
       </c>
-      <c r="G15" s="11" t="n">
+      <c r="G15" s="14" t="n">
         <v>20</v>
       </c>
-      <c r="H15" s="11" t="n">
+      <c r="H15" s="14" t="n">
         <v>11.75</v>
       </c>
-      <c r="I15" s="11"/>
-      <c r="J15" s="11" t="n">
+      <c r="I15" s="14"/>
+      <c r="J15" s="14" t="n">
         <v>7</v>
       </c>
-      <c r="K15" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="L15" s="11" t="n">
+      <c r="K15" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="L15" s="14" t="n">
         <f aca="false">SUM(B15:K15)</f>
         <v>67.5</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="11" t="s">
+    <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="14" t="s">
         <v>92</v>
       </c>
-      <c r="B16" s="11" t="n">
+      <c r="B16" s="14" t="n">
         <v>39.5</v>
       </c>
-      <c r="C16" s="11" t="n">
+      <c r="C16" s="14" t="n">
         <v>8</v>
       </c>
-      <c r="D16" s="11"/>
-      <c r="E16" s="11"/>
-      <c r="F16" s="11" t="n">
+      <c r="D16" s="14"/>
+      <c r="E16" s="14"/>
+      <c r="F16" s="14" t="n">
         <v>4.5</v>
       </c>
-      <c r="G16" s="11"/>
-      <c r="H16" s="11" t="n">
+      <c r="G16" s="14"/>
+      <c r="H16" s="14" t="n">
         <v>7.25</v>
       </c>
-      <c r="I16" s="11"/>
-      <c r="J16" s="11"/>
-      <c r="K16" s="11" t="n">
+      <c r="I16" s="14"/>
+      <c r="J16" s="14"/>
+      <c r="K16" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="L16" s="11" t="n">
+      <c r="L16" s="14" t="n">
         <f aca="false">SUM(B16:K16)</f>
         <v>63.25</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="11" t="s">
+    <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="14" t="s">
         <v>88</v>
       </c>
-      <c r="B17" s="11" t="n">
+      <c r="B17" s="14" t="n">
+        <f aca="false">3+11</f>
+        <v>14</v>
+      </c>
+      <c r="C17" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="D17" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="E17" s="14" t="n">
+        <v>16.75</v>
+      </c>
+      <c r="F17" s="14" t="n">
+        <f aca="false">1+1</f>
+        <v>2</v>
+      </c>
+      <c r="G17" s="14" t="n">
+        <f aca="false">17.75+29</f>
+        <v>46.75</v>
+      </c>
+      <c r="H17" s="14" t="n">
+        <f aca="false">2+7</f>
+        <v>9</v>
+      </c>
+      <c r="I17" s="14"/>
+      <c r="J17" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="C17" s="11" t="n">
-        <v>4</v>
-      </c>
-      <c r="D17" s="11"/>
-      <c r="E17" s="11" t="n">
-        <v>16.75</v>
-      </c>
-      <c r="F17" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="G17" s="11" t="n">
-        <v>17.75</v>
-      </c>
-      <c r="H17" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="I17" s="11"/>
-      <c r="J17" s="11" t="n">
+      <c r="K17" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="L17" s="14" t="n">
+        <f aca="false">SUM(B17:K17)</f>
+        <v>104.5</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="14" t="s">
+        <v>87</v>
+      </c>
+      <c r="B18" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="C18" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="D18" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="E18" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="F18" s="14"/>
+      <c r="G18" s="14" t="n">
+        <v>7</v>
+      </c>
+      <c r="H18" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="K17" s="11" t="n">
-        <v>5</v>
-      </c>
-      <c r="L17" s="11" t="n">
-        <f aca="false">SUM(B17:K17)</f>
-        <v>52.5</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="11" t="s">
-        <v>87</v>
-      </c>
-      <c r="B18" s="11" t="n">
-        <v>5</v>
-      </c>
-      <c r="C18" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="D18" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="E18" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="F18" s="11"/>
-      <c r="G18" s="11" t="n">
-        <v>7</v>
-      </c>
-      <c r="H18" s="11" t="n">
-        <v>3</v>
-      </c>
-      <c r="I18" s="11"/>
-      <c r="J18" s="11" t="n">
+      <c r="I18" s="14"/>
+      <c r="J18" s="14" t="n">
         <v>17.5</v>
       </c>
-      <c r="K18" s="11" t="n">
+      <c r="K18" s="14" t="n">
         <v>4.5</v>
       </c>
-      <c r="L18" s="11" t="n">
+      <c r="L18" s="14" t="n">
         <f aca="false">SUM(B18:K18)</f>
         <v>40</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="11" t="s">
+    <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="14" t="s">
         <v>93</v>
       </c>
-      <c r="B19" s="11" t="n">
+      <c r="B19" s="14" t="n">
         <v>4.5</v>
       </c>
-      <c r="C19" s="11" t="n">
+      <c r="C19" s="14" t="n">
         <v>10.5</v>
       </c>
-      <c r="D19" s="11" t="n">
+      <c r="D19" s="14" t="n">
         <v>8.75</v>
       </c>
-      <c r="E19" s="11"/>
-      <c r="F19" s="11" t="n">
+      <c r="E19" s="14"/>
+      <c r="F19" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="G19" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="H19" s="11"/>
-      <c r="I19" s="11"/>
-      <c r="J19" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="K19" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="L19" s="11" t="n">
+      <c r="G19" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="H19" s="14"/>
+      <c r="I19" s="14"/>
+      <c r="J19" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="K19" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="L19" s="14" t="n">
         <f aca="false">SUM(B19:K19)</f>
         <v>33.75</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="11" t="s">
+    <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="14" t="s">
         <v>95</v>
       </c>
-      <c r="B20" s="11" t="n">
+      <c r="B20" s="14" t="n">
         <v>12</v>
       </c>
-      <c r="C20" s="11"/>
-      <c r="D20" s="11"/>
-      <c r="E20" s="11"/>
-      <c r="F20" s="11"/>
-      <c r="G20" s="11"/>
-      <c r="H20" s="11" t="n">
+      <c r="C20" s="14"/>
+      <c r="D20" s="14"/>
+      <c r="E20" s="14"/>
+      <c r="F20" s="14"/>
+      <c r="G20" s="14"/>
+      <c r="H20" s="14" t="n">
         <v>9.75</v>
       </c>
-      <c r="I20" s="11" t="n">
+      <c r="I20" s="14" t="n">
         <v>11</v>
       </c>
-      <c r="J20" s="11"/>
-      <c r="K20" s="11" t="n">
+      <c r="J20" s="14"/>
+      <c r="K20" s="14" t="n">
         <v>0.25</v>
       </c>
-      <c r="L20" s="11" t="n">
+      <c r="L20" s="14" t="n">
         <f aca="false">SUM(B20:K20)</f>
         <v>33</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="11" t="s">
+    <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="14" t="s">
         <v>97</v>
       </c>
-      <c r="B21" s="11"/>
-      <c r="C21" s="11"/>
-      <c r="D21" s="11" t="n">
+      <c r="B21" s="14"/>
+      <c r="C21" s="14"/>
+      <c r="D21" s="14" t="n">
         <v>24.25</v>
       </c>
-      <c r="E21" s="11"/>
-      <c r="F21" s="11"/>
-      <c r="G21" s="11" t="n">
+      <c r="E21" s="14"/>
+      <c r="F21" s="14"/>
+      <c r="G21" s="14" t="n">
         <v>8</v>
       </c>
-      <c r="H21" s="11"/>
-      <c r="I21" s="11"/>
-      <c r="J21" s="11"/>
-      <c r="K21" s="11"/>
-      <c r="L21" s="11" t="n">
+      <c r="H21" s="14"/>
+      <c r="I21" s="14"/>
+      <c r="J21" s="14"/>
+      <c r="K21" s="14"/>
+      <c r="L21" s="14" t="n">
         <f aca="false">SUM(B21:K21)</f>
         <v>32.25</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="11" t="s">
+    <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="14" t="s">
         <v>94</v>
       </c>
-      <c r="B22" s="11"/>
-      <c r="C22" s="11"/>
-      <c r="D22" s="11" t="n">
+      <c r="B22" s="14"/>
+      <c r="C22" s="14"/>
+      <c r="D22" s="14" t="n">
         <v>13</v>
       </c>
-      <c r="E22" s="11"/>
-      <c r="F22" s="11"/>
-      <c r="G22" s="11" t="n">
+      <c r="E22" s="14"/>
+      <c r="F22" s="14"/>
+      <c r="G22" s="14" t="n">
         <v>11</v>
       </c>
-      <c r="H22" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="I22" s="11"/>
-      <c r="J22" s="11" t="n">
+      <c r="H22" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="I22" s="14"/>
+      <c r="J22" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="K22" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="L22" s="11" t="n">
+      <c r="K22" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="L22" s="14" t="n">
         <f aca="false">SUM(B22:K22)</f>
         <v>31</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="11" t="s">
+    <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="14" t="s">
         <v>90</v>
       </c>
-      <c r="B23" s="11"/>
-      <c r="C23" s="11" t="n">
+      <c r="B23" s="14"/>
+      <c r="C23" s="14" t="n">
         <v>3.5</v>
       </c>
-      <c r="D23" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="E23" s="11"/>
-      <c r="F23" s="11" t="n">
+      <c r="D23" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="E23" s="14"/>
+      <c r="F23" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="G23" s="11" t="n">
+      <c r="G23" s="14" t="n">
         <v>1.5</v>
       </c>
-      <c r="H23" s="11" t="n">
+      <c r="H23" s="14" t="n">
         <v>13</v>
       </c>
-      <c r="I23" s="11"/>
-      <c r="J23" s="11" t="n">
+      <c r="I23" s="14"/>
+      <c r="J23" s="14" t="n">
         <v>1.75</v>
       </c>
-      <c r="K23" s="11" t="n">
+      <c r="K23" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="L23" s="11" t="n">
+      <c r="L23" s="14" t="n">
         <f aca="false">SUM(B23:K23)</f>
         <v>25.75</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="11" t="s">
+    <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="14" t="s">
         <v>96</v>
       </c>
-      <c r="B24" s="11"/>
-      <c r="C24" s="11"/>
-      <c r="D24" s="11"/>
-      <c r="E24" s="11"/>
-      <c r="F24" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="G24" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="H24" s="11"/>
-      <c r="I24" s="11"/>
-      <c r="J24" s="11"/>
-      <c r="K24" s="11" t="n">
+      <c r="B24" s="14"/>
+      <c r="C24" s="14"/>
+      <c r="D24" s="14"/>
+      <c r="E24" s="14"/>
+      <c r="F24" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="G24" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="H24" s="14"/>
+      <c r="I24" s="14"/>
+      <c r="J24" s="14"/>
+      <c r="K24" s="14" t="n">
         <v>10</v>
       </c>
-      <c r="L24" s="11" t="n">
+      <c r="L24" s="14" t="n">
         <f aca="false">SUM(B24:K24)</f>
         <v>12</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="11" t="s">
+    <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="14" t="s">
         <v>98</v>
       </c>
-      <c r="B25" s="11"/>
-      <c r="C25" s="11" t="n">
+      <c r="B25" s="14"/>
+      <c r="C25" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="D25" s="11" t="n">
+      <c r="D25" s="14" t="n">
         <v>6.5</v>
       </c>
-      <c r="E25" s="11"/>
-      <c r="F25" s="11"/>
-      <c r="G25" s="11"/>
-      <c r="H25" s="11"/>
-      <c r="I25" s="11"/>
-      <c r="J25" s="11"/>
-      <c r="K25" s="11"/>
-      <c r="L25" s="11" t="n">
+      <c r="E25" s="14"/>
+      <c r="F25" s="14"/>
+      <c r="G25" s="14"/>
+      <c r="H25" s="14"/>
+      <c r="I25" s="14"/>
+      <c r="J25" s="14"/>
+      <c r="K25" s="14"/>
+      <c r="L25" s="14" t="n">
         <f aca="false">SUM(B25:K25)</f>
         <v>11.5</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="11" t="s">
+    <row r="26" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="14" t="s">
         <v>99</v>
       </c>
-      <c r="B26" s="11"/>
-      <c r="C26" s="11"/>
-      <c r="D26" s="11"/>
-      <c r="E26" s="11"/>
-      <c r="F26" s="11"/>
-      <c r="G26" s="11"/>
-      <c r="H26" s="11"/>
-      <c r="I26" s="11" t="n">
+      <c r="B26" s="14"/>
+      <c r="C26" s="14"/>
+      <c r="D26" s="14"/>
+      <c r="E26" s="14"/>
+      <c r="F26" s="14"/>
+      <c r="G26" s="14"/>
+      <c r="H26" s="14"/>
+      <c r="I26" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="J26" s="11" t="n">
+      <c r="J26" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="K26" s="11"/>
-      <c r="L26" s="11" t="n">
+      <c r="K26" s="14"/>
+      <c r="L26" s="14" t="n">
         <f aca="false">SUM(B26:K26)</f>
         <v>10</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="11" t="s">
+    <row r="27" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="14" t="s">
         <v>100</v>
       </c>
-      <c r="B27" s="11"/>
-      <c r="C27" s="11"/>
-      <c r="D27" s="11"/>
-      <c r="E27" s="11"/>
-      <c r="F27" s="11"/>
-      <c r="G27" s="11"/>
-      <c r="H27" s="11"/>
-      <c r="I27" s="11"/>
-      <c r="J27" s="11"/>
-      <c r="K27" s="11" t="n">
+      <c r="B27" s="14"/>
+      <c r="C27" s="14"/>
+      <c r="D27" s="14"/>
+      <c r="E27" s="14"/>
+      <c r="F27" s="14"/>
+      <c r="G27" s="14"/>
+      <c r="H27" s="14"/>
+      <c r="I27" s="14"/>
+      <c r="J27" s="14"/>
+      <c r="K27" s="14" t="n">
         <v>3.5</v>
       </c>
-      <c r="L27" s="11" t="n">
+      <c r="L27" s="14" t="n">
         <f aca="false">SUM(B27:K27)</f>
         <v>3.5</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="7" t="s">
+    <row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="14" t="s">
+        <v>101</v>
+      </c>
+      <c r="B28" s="14" t="n">
+        <v>73</v>
+      </c>
+      <c r="C28" s="14" t="n">
+        <v>241</v>
+      </c>
+      <c r="D28" s="14" t="n">
+        <v>209</v>
+      </c>
+      <c r="E28" s="14" t="n">
+        <v>88</v>
+      </c>
+      <c r="F28" s="14" t="n">
+        <v>59</v>
+      </c>
+      <c r="G28" s="14" t="n">
+        <v>121</v>
+      </c>
+      <c r="H28" s="14" t="n">
+        <v>22</v>
+      </c>
+      <c r="I28" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="J28" s="14" t="n">
+        <v>28</v>
+      </c>
+      <c r="K28" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="L28" s="14" t="n">
+        <f aca="false">SUM(B28:K28)</f>
+        <v>846</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="7" t="s">
         <v>74</v>
       </c>
-      <c r="B28" s="7" t="n">
-        <f aca="false">SUM(B4:B27)</f>
-        <v>675.5</v>
-      </c>
-      <c r="C28" s="7" t="n">
-        <f aca="false">SUM(C4:C27)</f>
-        <v>627.25</v>
-      </c>
-      <c r="D28" s="7" t="n">
-        <f aca="false">SUM(D4:D27)</f>
-        <v>578.25</v>
-      </c>
-      <c r="E28" s="7" t="n">
-        <f aca="false">SUM(E4:E27)</f>
-        <v>572.05</v>
-      </c>
-      <c r="F28" s="7" t="n">
-        <f aca="false">SUM(F4:F27)</f>
-        <v>587.25</v>
-      </c>
-      <c r="G28" s="7" t="n">
-        <f aca="false">SUM(G4:G27)</f>
-        <v>668.3</v>
-      </c>
-      <c r="H28" s="7" t="n">
-        <f aca="false">SUM(H4:H27)</f>
-        <v>660.9</v>
-      </c>
-      <c r="I28" s="7" t="n">
-        <f aca="false">SUM(I4:I27)</f>
+      <c r="B29" s="7" t="n">
+        <f aca="false">SUM(B4:B28)</f>
+        <v>780.5</v>
+      </c>
+      <c r="C29" s="7" t="n">
+        <f aca="false">SUM(C4:C28)</f>
+        <v>872.25</v>
+      </c>
+      <c r="D29" s="7" t="n">
+        <f aca="false">SUM(D4:D28)</f>
+        <v>824.25</v>
+      </c>
+      <c r="E29" s="7" t="n">
+        <f aca="false">SUM(E4:E28)</f>
+        <v>673.05</v>
+      </c>
+      <c r="F29" s="7" t="n">
+        <f aca="false">SUM(F4:F28)</f>
+        <v>694.25</v>
+      </c>
+      <c r="G29" s="7" t="n">
+        <f aca="false">SUM(G4:G28)</f>
+        <v>837.3</v>
+      </c>
+      <c r="H29" s="7" t="n">
+        <f aca="false">SUM(H4:H28)</f>
+        <v>712.9</v>
+      </c>
+      <c r="I29" s="7" t="n">
+        <f aca="false">SUM(I4:I28)</f>
         <v>437.25</v>
       </c>
-      <c r="J28" s="7" t="n">
-        <f aca="false">SUM(J4:J27)</f>
-        <v>726.25</v>
-      </c>
-      <c r="K28" s="7" t="n">
-        <f aca="false">SUM(K4:K27)</f>
-        <v>385.25</v>
-      </c>
-      <c r="L28" s="7" t="n">
-        <f aca="false">SUM(L4:L27)</f>
-        <v>5918.25</v>
+      <c r="J29" s="7" t="n">
+        <f aca="false">SUM(J4:J28)</f>
+        <v>755.25</v>
+      </c>
+      <c r="K29" s="7" t="n">
+        <f aca="false">SUM(K4:K28)</f>
+        <v>390.25</v>
+      </c>
+      <c r="L29" s="7" t="n">
+        <f aca="false">SUM(L4:L28)</f>
+        <v>6977.25</v>
       </c>
     </row>
   </sheetData>
@@ -3617,29 +3829,29 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:L10"/>
-  <sheetFormatPr defaultColWidth="8.66796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.66796875" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="2" style="0" width="14"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="10" t="s">
-        <v>102</v>
-      </c>
-      <c r="B1" s="10"/>
-      <c r="C1" s="10"/>
-      <c r="D1" s="10"/>
-      <c r="E1" s="10"/>
-      <c r="F1" s="10"/>
-      <c r="G1" s="10"/>
-      <c r="H1" s="10"/>
-      <c r="I1" s="10"/>
-      <c r="J1" s="10"/>
-      <c r="K1" s="10"/>
-      <c r="L1" s="10"/>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="15" t="s">
+        <v>103</v>
+      </c>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="15"/>
+      <c r="G1" s="15"/>
+      <c r="H1" s="15"/>
+      <c r="I1" s="15"/>
+      <c r="J1" s="15"/>
+      <c r="K1" s="15"/>
+      <c r="L1" s="15"/>
+    </row>
+    <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
         <v>41</v>
       </c>
@@ -3677,215 +3889,215 @@
         <v>59</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="11" t="s">
-        <v>103</v>
-      </c>
-      <c r="B4" s="11" t="n">
+    <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="16" t="s">
+        <v>104</v>
+      </c>
+      <c r="B4" s="16" t="n">
         <v>77</v>
       </c>
-      <c r="C4" s="11" t="n">
+      <c r="C4" s="16" t="n">
         <v>73</v>
       </c>
-      <c r="D4" s="11" t="n">
+      <c r="D4" s="16" t="n">
         <v>66</v>
       </c>
-      <c r="E4" s="11" t="n">
+      <c r="E4" s="16" t="n">
         <v>57</v>
       </c>
-      <c r="F4" s="11" t="n">
+      <c r="F4" s="16" t="n">
         <v>87</v>
       </c>
-      <c r="G4" s="11" t="n">
+      <c r="G4" s="16" t="n">
         <v>97</v>
       </c>
-      <c r="H4" s="11" t="n">
+      <c r="H4" s="16" t="n">
         <v>106</v>
       </c>
-      <c r="I4" s="11" t="n">
+      <c r="I4" s="16" t="n">
         <v>25</v>
       </c>
-      <c r="J4" s="11" t="n">
+      <c r="J4" s="16" t="n">
         <v>76</v>
       </c>
-      <c r="K4" s="11" t="n">
+      <c r="K4" s="16" t="n">
         <v>87</v>
       </c>
-      <c r="L4" s="11" t="n">
+      <c r="L4" s="16" t="n">
         <f aca="false">SUM(B4:K4)</f>
         <v>751</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="11" t="s">
-        <v>104</v>
-      </c>
-      <c r="B5" s="11" t="n">
+    <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="16" t="s">
+        <v>105</v>
+      </c>
+      <c r="B5" s="16" t="n">
         <v>27</v>
       </c>
-      <c r="C5" s="11" t="n">
+      <c r="C5" s="16" t="n">
         <v>14</v>
       </c>
-      <c r="D5" s="11" t="n">
+      <c r="D5" s="16" t="n">
         <v>18</v>
       </c>
-      <c r="E5" s="11" t="n">
+      <c r="E5" s="16" t="n">
         <v>15</v>
       </c>
-      <c r="F5" s="11" t="n">
+      <c r="F5" s="16" t="n">
         <v>10</v>
       </c>
-      <c r="G5" s="11" t="n">
+      <c r="G5" s="16" t="n">
         <v>36</v>
       </c>
-      <c r="H5" s="11" t="n">
+      <c r="H5" s="16" t="n">
         <v>12</v>
       </c>
-      <c r="I5" s="11" t="n">
+      <c r="I5" s="16" t="n">
         <v>3</v>
       </c>
-      <c r="J5" s="11" t="n">
+      <c r="J5" s="16" t="n">
         <v>9</v>
       </c>
-      <c r="K5" s="11" t="n">
+      <c r="K5" s="16" t="n">
         <v>11</v>
       </c>
-      <c r="L5" s="11" t="n">
+      <c r="L5" s="16" t="n">
         <f aca="false">SUM(B5:K5)</f>
         <v>155</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="11" t="s">
-        <v>105</v>
-      </c>
-      <c r="B6" s="11" t="n">
+    <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="16" t="s">
+        <v>106</v>
+      </c>
+      <c r="B6" s="16" t="n">
         <v>4</v>
       </c>
-      <c r="C6" s="11" t="n">
+      <c r="C6" s="16" t="n">
         <v>13</v>
       </c>
-      <c r="D6" s="11" t="n">
+      <c r="D6" s="16" t="n">
         <v>4</v>
       </c>
-      <c r="E6" s="11" t="n">
+      <c r="E6" s="16" t="n">
         <v>16</v>
       </c>
-      <c r="F6" s="11" t="n">
+      <c r="F6" s="16" t="n">
         <v>13</v>
       </c>
-      <c r="G6" s="11" t="n">
+      <c r="G6" s="16" t="n">
         <v>13</v>
       </c>
-      <c r="H6" s="11" t="n">
+      <c r="H6" s="16" t="n">
         <v>13</v>
       </c>
-      <c r="I6" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="J6" s="11" t="n">
+      <c r="I6" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="J6" s="16" t="n">
         <v>24</v>
       </c>
-      <c r="K6" s="11" t="n">
+      <c r="K6" s="16" t="n">
         <v>36</v>
       </c>
-      <c r="L6" s="11" t="n">
+      <c r="L6" s="16" t="n">
         <f aca="false">SUM(B6:K6)</f>
         <v>138</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="11" t="s">
-        <v>106</v>
-      </c>
-      <c r="B7" s="11"/>
-      <c r="C7" s="11" t="n">
+    <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="16" t="s">
+        <v>107</v>
+      </c>
+      <c r="B7" s="16"/>
+      <c r="C7" s="16" t="n">
         <v>5</v>
       </c>
-      <c r="D7" s="11" t="n">
+      <c r="D7" s="16" t="n">
         <v>3</v>
       </c>
-      <c r="E7" s="11"/>
-      <c r="F7" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="G7" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="H7" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="I7" s="11"/>
-      <c r="J7" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="K7" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="L7" s="11" t="n">
+      <c r="E7" s="16"/>
+      <c r="F7" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="G7" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="H7" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="I7" s="16"/>
+      <c r="J7" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="K7" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="L7" s="16" t="n">
         <f aca="false">SUM(B7:K7)</f>
         <v>13</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="11" t="s">
-        <v>107</v>
-      </c>
-      <c r="B8" s="11"/>
-      <c r="C8" s="11"/>
-      <c r="D8" s="11"/>
-      <c r="E8" s="11"/>
-      <c r="F8" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="G8" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="H8" s="11" t="n">
+    <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="16" t="s">
+        <v>108</v>
+      </c>
+      <c r="B8" s="16"/>
+      <c r="C8" s="16"/>
+      <c r="D8" s="16"/>
+      <c r="E8" s="16"/>
+      <c r="F8" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="G8" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="H8" s="16" t="n">
         <v>4</v>
       </c>
-      <c r="I8" s="11"/>
-      <c r="J8" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="K8" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="L8" s="11" t="n">
+      <c r="I8" s="16"/>
+      <c r="J8" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="K8" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="L8" s="16" t="n">
         <f aca="false">SUM(B8:K8)</f>
         <v>10</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="11" t="s">
-        <v>108</v>
-      </c>
-      <c r="B9" s="11" t="n">
+    <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="16" t="s">
+        <v>109</v>
+      </c>
+      <c r="B9" s="16" t="n">
         <v>3</v>
       </c>
-      <c r="C9" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="D9" s="11"/>
-      <c r="E9" s="11"/>
-      <c r="F9" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="G9" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="H9" s="11"/>
-      <c r="I9" s="11"/>
-      <c r="J9" s="11"/>
-      <c r="K9" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="L9" s="11" t="n">
+      <c r="C9" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="D9" s="16"/>
+      <c r="E9" s="16"/>
+      <c r="F9" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="G9" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="H9" s="16"/>
+      <c r="I9" s="16"/>
+      <c r="J9" s="16"/>
+      <c r="K9" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="L9" s="16" t="n">
         <f aca="false">SUM(B9:K9)</f>
         <v>10</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
         <v>74</v>
       </c>
@@ -3954,7 +4166,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:K6"/>
-  <sheetFormatPr defaultColWidth="8.66796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.66796875" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="28"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="2" style="0" width="14"/>
@@ -3962,7 +4174,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="10" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B1" s="10"/>
       <c r="C1" s="10"/>
@@ -3975,9 +4187,9 @@
       <c r="J1" s="10"/>
       <c r="K1" s="10"/>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B3" s="7" t="s">
         <v>49</v>
@@ -4010,73 +4222,81 @@
         <v>58</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="13" t="s">
-        <v>111</v>
-      </c>
-      <c r="B4" s="11" t="n">
+    <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="17" t="s">
+        <v>112</v>
+      </c>
+      <c r="B4" s="14" t="n">
         <v>2.03</v>
       </c>
-      <c r="C4" s="11" t="n">
+      <c r="C4" s="14" t="n">
         <v>2.38</v>
       </c>
-      <c r="D4" s="11" t="n">
+      <c r="D4" s="14" t="n">
         <v>2.35</v>
       </c>
-      <c r="E4" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="F4" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="G4" s="11"/>
-      <c r="H4" s="11"/>
-      <c r="I4" s="11"/>
-      <c r="J4" s="11"/>
-      <c r="K4" s="11"/>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="13" t="s">
-        <v>112</v>
-      </c>
-      <c r="B5" s="11" t="n">
-        <v>2.06</v>
-      </c>
-      <c r="C5" s="11" t="n">
-        <v>1.84</v>
-      </c>
-      <c r="D5" s="11" t="n">
-        <v>1.63</v>
-      </c>
-      <c r="E5" s="11" t="n">
+      <c r="E4" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="F4" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="G4" s="14"/>
+      <c r="H4" s="14"/>
+      <c r="I4" s="14"/>
+      <c r="J4" s="14"/>
+      <c r="K4" s="14"/>
+    </row>
+    <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="17" t="s">
+        <v>101</v>
+      </c>
+      <c r="B5" s="14" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="C5" s="14" t="n">
         <v>1.7</v>
       </c>
-      <c r="F5" s="11" t="n">
-        <v>1.6</v>
-      </c>
-      <c r="G5" s="11"/>
-      <c r="H5" s="11"/>
-      <c r="I5" s="11"/>
-      <c r="J5" s="11"/>
-      <c r="K5" s="11"/>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D5" s="14" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="E5" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="G5" s="14" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="H5" s="14" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="I5" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" s="14" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="K5" s="14"/>
+    </row>
+    <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
         <v>113</v>
       </c>
-      <c r="B6" s="14" t="n">
+      <c r="B6" s="18" t="n">
         <f aca="false">AVERAGE(B4:K5)</f>
-        <v>1.959</v>
-      </c>
-      <c r="C6" s="14"/>
-      <c r="D6" s="14"/>
-      <c r="E6" s="14"/>
-      <c r="F6" s="14"/>
-      <c r="G6" s="14"/>
-      <c r="H6" s="14"/>
-      <c r="I6" s="14"/>
-      <c r="J6" s="14"/>
-      <c r="K6" s="14"/>
+        <v>1.69</v>
+      </c>
+      <c r="C6" s="18"/>
+      <c r="D6" s="18"/>
+      <c r="E6" s="18"/>
+      <c r="F6" s="18"/>
+      <c r="G6" s="18"/>
+      <c r="H6" s="18"/>
+      <c r="I6" s="18"/>
+      <c r="J6" s="18"/>
+      <c r="K6" s="18"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -4099,7 +4319,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:L5"/>
-  <sheetFormatPr defaultColWidth="8.66796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.66796875" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="28"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="2" style="0" width="14"/>
@@ -4121,9 +4341,9 @@
       <c r="K1" s="10"/>
       <c r="L1" s="10"/>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B3" s="7" t="s">
         <v>49</v>
@@ -4159,82 +4379,93 @@
         <v>59</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="13" t="s">
+    <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="17" t="s">
         <v>115</v>
       </c>
-      <c r="B4" s="11" t="n">
-        <v>25</v>
-      </c>
-      <c r="C4" s="11" t="n">
+      <c r="B4" s="14" t="n">
+        <f aca="false">25+1</f>
+        <v>26</v>
+      </c>
+      <c r="C4" s="14" t="n">
         <v>21</v>
       </c>
-      <c r="D4" s="11" t="n">
-        <v>22</v>
-      </c>
-      <c r="E4" s="11" t="n">
+      <c r="D4" s="14" t="n">
+        <f aca="false">22+1</f>
+        <v>23</v>
+      </c>
+      <c r="E4" s="14" t="n">
         <v>7</v>
       </c>
-      <c r="F4" s="11" t="n">
+      <c r="F4" s="14" t="n">
         <v>19</v>
       </c>
-      <c r="G4" s="11" t="n">
-        <v>29</v>
-      </c>
-      <c r="H4" s="11" t="n">
-        <v>36</v>
-      </c>
-      <c r="I4" s="11" t="n">
+      <c r="G4" s="14" t="n">
+        <f aca="false">29+1</f>
+        <v>30</v>
+      </c>
+      <c r="H4" s="14" t="n">
+        <f aca="false">36+1</f>
+        <v>37</v>
+      </c>
+      <c r="I4" s="14" t="n">
         <v>7</v>
       </c>
-      <c r="J4" s="11" t="n">
-        <v>16</v>
-      </c>
-      <c r="K4" s="11" t="n">
-        <v>22</v>
-      </c>
-      <c r="L4" s="11" t="n">
+      <c r="J4" s="14" t="n">
+        <f aca="false">16+1</f>
+        <v>17</v>
+      </c>
+      <c r="K4" s="14" t="n">
+        <f aca="false">22+1</f>
+        <v>23</v>
+      </c>
+      <c r="L4" s="14" t="n">
         <f aca="false">SUM(B4:K4)</f>
-        <v>204</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="13" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="17" t="s">
         <v>116</v>
       </c>
-      <c r="B5" s="11" t="n">
-        <v>13.75</v>
-      </c>
-      <c r="C5" s="11" t="n">
+      <c r="B5" s="14" t="n">
+        <f aca="false">13.75+12</f>
+        <v>25.75</v>
+      </c>
+      <c r="C5" s="14" t="n">
         <v>23.25</v>
       </c>
-      <c r="D5" s="11" t="n">
-        <v>19</v>
-      </c>
-      <c r="E5" s="11" t="n">
+      <c r="D5" s="14" t="n">
+        <f aca="false">19+16</f>
+        <v>35</v>
+      </c>
+      <c r="E5" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="F5" s="11" t="n">
+      <c r="F5" s="14" t="n">
         <v>12.25</v>
       </c>
-      <c r="G5" s="11" t="n">
-        <v>14.55</v>
-      </c>
-      <c r="H5" s="11" t="n">
-        <v>30.6</v>
-      </c>
-      <c r="I5" s="11" t="n">
+      <c r="G5" s="14" t="n">
+        <f aca="false">14.55+1</f>
+        <v>15.55</v>
+      </c>
+      <c r="H5" s="14" t="n">
+        <f aca="false">30.6+7</f>
+        <v>37.6</v>
+      </c>
+      <c r="I5" s="14" t="n">
         <v>12.75</v>
       </c>
-      <c r="J5" s="11" t="n">
-        <v>22</v>
-      </c>
-      <c r="K5" s="11" t="n">
+      <c r="J5" s="14" t="n">
+        <f aca="false">22+1</f>
+        <v>23</v>
+      </c>
+      <c r="K5" s="14" t="n">
         <v>8.5</v>
       </c>
-      <c r="L5" s="11" t="n">
+      <c r="L5" s="14" t="n">
         <f aca="false">SUM(B5:K5)</f>
-        <v>161.65</v>
+        <v>198.65</v>
       </c>
     </row>
   </sheetData>
@@ -4257,7 +4488,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:L4"/>
-  <sheetFormatPr defaultColWidth="11.5078125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.5625" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="13"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="2" style="0" width="14"/>
@@ -4279,7 +4510,7 @@
       <c r="K1" s="10"/>
       <c r="L1" s="10"/>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="7"/>
       <c r="B3" s="7" t="s">
         <v>49</v>
@@ -4315,43 +4546,43 @@
         <v>59</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="11" t="s">
+    <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="14" t="s">
         <v>118</v>
       </c>
-      <c r="B4" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="C4" s="11" t="n">
+      <c r="B4" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="C4" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="D4" s="11" t="n">
+      <c r="D4" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="E4" s="11" t="n">
+      <c r="E4" s="14" t="n">
         <v>8</v>
       </c>
-      <c r="F4" s="11" t="n">
+      <c r="F4" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="G4" s="11" t="n">
+      <c r="G4" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="H4" s="11" t="n">
+      <c r="H4" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="I4" s="11" t="n">
+      <c r="I4" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="J4" s="11" t="n">
+      <c r="J4" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="K4" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="K4" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="L4" s="11" t="n">
+      <c r="L4" s="14" t="n">
         <f aca="false">SUM(B4:K4)</f>
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualizar datos con datos 4.xlsx (incluye Retail) (#29)
Se publica el Excel "datos 4.xlsx" renombrado a datos.xlsx, con Retail en
Negocio_Volumen y Negocio_Horas, entrega de Retail hasta septiembre y un
freelance más en septiembre.

La hoja Ciudad se mantiene como estaba publicada: en la nueva, Madrid
febrero vale 73208 (falta "=" y "+") y las sumas añadidas a Madrid hacen
que las ciudades sumen el doble que el total de trabajos. Queda
pendiente de que se corrija en el Excel.


Claude-Session: https://claude.ai/code/session_01A4SLDFHLc22bTWoXT2NUrv

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Instrucciones" sheetId="1" state="visible" r:id="rId3"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="119">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="219" uniqueCount="119">
   <si>
     <t xml:space="preserve">PLANTILLA DASHBOARD BDESIGN</t>
   </si>
@@ -332,6 +332,9 @@
     <t xml:space="preserve">Foro Innovacion</t>
   </si>
   <si>
+    <t xml:space="preserve">Retail</t>
+  </si>
+  <si>
     <t xml:space="preserve">HORAS dedicadas por DEPARTAMENTO/NEGOCIO</t>
   </si>
   <si>
@@ -363,9 +366,6 @@
   </si>
   <si>
     <t xml:space="preserve">Bdesign</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Retail</t>
   </si>
   <si>
     <t xml:space="preserve">MEDIA YTD</t>
@@ -395,7 +395,7 @@
     <numFmt numFmtId="165" formatCode="General"/>
     <numFmt numFmtId="166" formatCode="0.0"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="14">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -471,6 +471,21 @@
       <charset val="1"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
@@ -492,7 +507,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
@@ -512,6 +527,21 @@
       </top>
       <bottom style="thin">
         <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="medium">
+        <color rgb="FFE6E6E6"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFE6E6E6"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFE6E6E6"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFE6E6E6"/>
       </bottom>
       <diagonal/>
     </border>
@@ -541,7 +571,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="19">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -586,12 +616,28 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
@@ -631,7 +677,7 @@
       <rgbColor rgb="FF808080"/>
       <rgbColor rgb="FF9999FF"/>
       <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FFFFFFCC"/>
+      <rgbColor rgb="FFE6E6E6"/>
       <rgbColor rgb="FFCCFFFF"/>
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
@@ -855,7 +901,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D37"/>
-  <sheetFormatPr defaultColWidth="8.66796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.66796875" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="24"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="2" style="0" width="28"/>
@@ -1151,7 +1197,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:L19"/>
-  <sheetFormatPr defaultColWidth="8.66796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.66796875" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="2" style="0" width="14"/>
@@ -1173,7 +1219,7 @@
       <c r="K1" s="10"/>
       <c r="L1" s="10"/>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
         <v>48</v>
       </c>
@@ -1211,57 +1257,57 @@
         <v>59</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="11" t="s">
         <v>60</v>
       </c>
       <c r="B4" s="11" t="n">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="C4" s="11" t="n">
-        <v>28</v>
+        <v>40</v>
       </c>
       <c r="D4" s="11" t="n">
-        <v>23</v>
+        <v>32</v>
       </c>
       <c r="E4" s="11" t="n">
-        <v>25</v>
+        <v>34</v>
       </c>
       <c r="F4" s="11" t="n">
-        <v>36</v>
+        <v>45</v>
       </c>
       <c r="G4" s="11" t="n">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="H4" s="11" t="n">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="I4" s="11" t="n">
         <v>10</v>
       </c>
       <c r="J4" s="11" t="n">
-        <v>41</v>
+        <v>52</v>
       </c>
       <c r="K4" s="11" t="n">
-        <v>48</v>
-      </c>
-      <c r="L4" s="11" t="n">
+        <v>55</v>
+      </c>
+      <c r="L4" s="12" t="n">
         <f aca="false">SUM(B4:K4)</f>
-        <v>307</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="11" t="s">
         <v>45</v>
       </c>
       <c r="B5" s="11" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C5" s="11" t="n">
         <v>21</v>
       </c>
       <c r="D5" s="11" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E5" s="11" t="n">
         <v>7</v>
@@ -1270,26 +1316,26 @@
         <v>19</v>
       </c>
       <c r="G5" s="11" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="H5" s="11" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="I5" s="11" t="n">
         <v>7</v>
       </c>
       <c r="J5" s="11" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="K5" s="11" t="n">
-        <v>22</v>
-      </c>
-      <c r="L5" s="11" t="n">
+        <v>23</v>
+      </c>
+      <c r="L5" s="12" t="n">
         <f aca="false">SUM(B5:K5)</f>
-        <v>204</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="11" t="s">
         <v>61</v>
       </c>
@@ -1303,89 +1349,91 @@
         <v>12</v>
       </c>
       <c r="E6" s="11" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="F6" s="11" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="G6" s="11" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="H6" s="11" t="n">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="I6" s="11" t="n">
         <v>2</v>
       </c>
       <c r="J6" s="11" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="K6" s="11" t="n">
         <v>31</v>
       </c>
-      <c r="L6" s="11" t="n">
+      <c r="L6" s="12" t="n">
         <f aca="false">SUM(B6:K6)</f>
-        <v>175</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="11" t="s">
         <v>62</v>
       </c>
       <c r="B7" s="11" t="n">
+        <v>16</v>
+      </c>
+      <c r="C7" s="11" t="n">
         <v>14</v>
       </c>
-      <c r="C7" s="11" t="n">
-        <v>8</v>
-      </c>
       <c r="D7" s="11" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E7" s="11" t="n">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="F7" s="11" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="G7" s="11" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="H7" s="11" t="n">
-        <v>10</v>
-      </c>
-      <c r="I7" s="11"/>
+        <v>15</v>
+      </c>
+      <c r="I7" s="11" t="n">
+        <v>0</v>
+      </c>
       <c r="J7" s="11" t="n">
         <v>4</v>
       </c>
       <c r="K7" s="11" t="n">
-        <v>8</v>
-      </c>
-      <c r="L7" s="11" t="n">
+        <v>9</v>
+      </c>
+      <c r="L7" s="12" t="n">
         <f aca="false">SUM(B7:K7)</f>
-        <v>83</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="11" t="s">
         <v>63</v>
       </c>
       <c r="B8" s="11" t="n">
+        <v>11</v>
+      </c>
+      <c r="C8" s="11" t="n">
+        <v>7</v>
+      </c>
+      <c r="D8" s="11" t="n">
         <v>9</v>
-      </c>
-      <c r="C8" s="11" t="n">
-        <v>6</v>
-      </c>
-      <c r="D8" s="11" t="n">
-        <v>6</v>
       </c>
       <c r="E8" s="11" t="n">
         <v>10</v>
       </c>
       <c r="F8" s="11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G8" s="11" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="H8" s="11" t="n">
         <v>5</v>
@@ -1394,17 +1442,17 @@
         <v>3</v>
       </c>
       <c r="J8" s="11" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="K8" s="11" t="n">
-        <v>6</v>
-      </c>
-      <c r="L8" s="11" t="n">
+        <v>7</v>
+      </c>
+      <c r="L8" s="12" t="n">
         <f aca="false">SUM(B8:K8)</f>
-        <v>67</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="11" t="s">
         <v>64</v>
       </c>
@@ -1433,93 +1481,95 @@
         <v>2</v>
       </c>
       <c r="J9" s="11" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="K9" s="11" t="n">
         <v>5</v>
       </c>
-      <c r="L9" s="11" t="n">
+      <c r="L9" s="12" t="n">
         <f aca="false">SUM(B9:K9)</f>
-        <v>58</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="11" t="s">
         <v>65</v>
       </c>
       <c r="B10" s="11" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C10" s="11" t="n">
+        <v>9</v>
+      </c>
+      <c r="D10" s="11" t="n">
+        <v>7</v>
+      </c>
+      <c r="E10" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="D10" s="11" t="n">
+      <c r="F10" s="11" t="n">
         <v>6</v>
       </c>
-      <c r="E10" s="11" t="n">
+      <c r="G10" s="11" t="n">
         <v>6</v>
       </c>
-      <c r="F10" s="11" t="n">
-        <v>3</v>
-      </c>
-      <c r="G10" s="11" t="n">
-        <v>5</v>
-      </c>
       <c r="H10" s="11" t="n">
-        <v>11</v>
-      </c>
-      <c r="I10" s="11"/>
+        <v>13</v>
+      </c>
+      <c r="I10" s="11" t="n">
+        <v>0</v>
+      </c>
       <c r="J10" s="11" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="K10" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="L10" s="11" t="n">
+      <c r="L10" s="12" t="n">
         <f aca="false">SUM(B10:K10)</f>
-        <v>53</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="11" t="s">
         <v>66</v>
       </c>
       <c r="B11" s="11" t="n">
+        <v>10</v>
+      </c>
+      <c r="C11" s="11" t="n">
+        <v>10</v>
+      </c>
+      <c r="D11" s="11" t="n">
+        <v>7</v>
+      </c>
+      <c r="E11" s="11" t="n">
+        <v>5</v>
+      </c>
+      <c r="F11" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="G11" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="H11" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="I11" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="J11" s="11" t="n">
+        <v>11</v>
+      </c>
+      <c r="K11" s="11" t="n">
         <v>9</v>
       </c>
-      <c r="C11" s="11" t="n">
-        <v>4</v>
-      </c>
-      <c r="D11" s="11" t="n">
-        <v>4</v>
-      </c>
-      <c r="E11" s="11" t="n">
-        <v>3</v>
-      </c>
-      <c r="F11" s="11" t="n">
-        <v>3</v>
-      </c>
-      <c r="G11" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="H11" s="11" t="n">
-        <v>3</v>
-      </c>
-      <c r="I11" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="J11" s="11" t="n">
-        <v>7</v>
-      </c>
-      <c r="K11" s="11" t="n">
-        <v>3</v>
-      </c>
-      <c r="L11" s="11" t="n">
+      <c r="L11" s="12" t="n">
         <f aca="false">SUM(B11:K11)</f>
-        <v>40</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="11" t="s">
         <v>67</v>
       </c>
@@ -1529,8 +1579,12 @@
       <c r="C12" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="D12" s="11"/>
-      <c r="E12" s="11"/>
+      <c r="D12" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" s="11" t="n">
+        <v>0</v>
+      </c>
       <c r="F12" s="11" t="n">
         <v>7</v>
       </c>
@@ -1538,66 +1592,74 @@
         <v>4</v>
       </c>
       <c r="H12" s="11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I12" s="11" t="n">
         <v>2</v>
       </c>
       <c r="J12" s="11" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="K12" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="L12" s="11" t="n">
+      <c r="L12" s="12" t="n">
         <f aca="false">SUM(B12:K12)</f>
-        <v>26</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="11" t="s">
         <v>68</v>
       </c>
       <c r="B13" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="C13" s="11"/>
-      <c r="D13" s="11"/>
+      <c r="C13" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13" s="11" t="n">
+        <v>2</v>
+      </c>
       <c r="E13" s="11" t="n">
         <v>1</v>
       </c>
       <c r="F13" s="11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G13" s="11" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H13" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="I13" s="11"/>
+        <v>6</v>
+      </c>
+      <c r="I13" s="11" t="n">
+        <v>0</v>
+      </c>
       <c r="J13" s="11" t="n">
         <v>1</v>
       </c>
       <c r="K13" s="11" t="n">
         <v>6</v>
       </c>
-      <c r="L13" s="11" t="n">
+      <c r="L13" s="12" t="n">
         <f aca="false">SUM(B13:K13)</f>
-        <v>18</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="11" t="s">
         <v>69</v>
       </c>
       <c r="B14" s="11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C14" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="D14" s="11"/>
+      <c r="D14" s="11" t="n">
+        <v>0</v>
+      </c>
       <c r="E14" s="11" t="n">
         <v>3</v>
       </c>
@@ -1605,31 +1667,37 @@
         <v>2</v>
       </c>
       <c r="G14" s="11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H14" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="I14" s="11"/>
+      <c r="I14" s="11" t="n">
+        <v>0</v>
+      </c>
       <c r="J14" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="K14" s="11"/>
-      <c r="L14" s="11" t="n">
+      <c r="K14" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" s="12" t="n">
         <f aca="false">SUM(B14:K14)</f>
-        <v>16</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="11" t="s">
         <v>70</v>
       </c>
       <c r="B15" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="C15" s="11"/>
+      <c r="C15" s="11" t="n">
+        <v>0</v>
+      </c>
       <c r="D15" s="11" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E15" s="11" t="n">
         <v>2</v>
@@ -1638,62 +1706,86 @@
         <v>1</v>
       </c>
       <c r="G15" s="11" t="n">
-        <v>4</v>
-      </c>
-      <c r="H15" s="11"/>
-      <c r="I15" s="11"/>
-      <c r="J15" s="11"/>
+        <v>5</v>
+      </c>
+      <c r="H15" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J15" s="11" t="n">
+        <v>0</v>
+      </c>
       <c r="K15" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="L15" s="11" t="n">
+      <c r="L15" s="12" t="n">
         <f aca="false">SUM(B15:K15)</f>
-        <v>14</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="11" t="s">
         <v>71</v>
       </c>
       <c r="B16" s="11" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C16" s="11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D16" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="E16" s="11"/>
-      <c r="F16" s="11"/>
+        <v>4</v>
+      </c>
+      <c r="E16" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F16" s="11" t="n">
+        <v>0</v>
+      </c>
       <c r="G16" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="H16" s="11"/>
+        <v>2</v>
+      </c>
+      <c r="H16" s="11" t="n">
+        <v>0</v>
+      </c>
       <c r="I16" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="J16" s="11"/>
+      <c r="J16" s="11" t="n">
+        <v>3</v>
+      </c>
       <c r="K16" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="L16" s="11" t="n">
+      <c r="L16" s="12" t="n">
         <f aca="false">SUM(B16:K16)</f>
-        <v>10</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="11" t="s">
         <v>72</v>
       </c>
-      <c r="B17" s="11"/>
-      <c r="C17" s="11"/>
-      <c r="D17" s="11"/>
+      <c r="B17" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D17" s="11" t="n">
+        <v>1</v>
+      </c>
       <c r="E17" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="F17" s="11"/>
-      <c r="G17" s="11"/>
+      <c r="F17" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" s="11" t="n">
+        <v>2</v>
+      </c>
       <c r="H17" s="11" t="n">
         <v>1</v>
       </c>
@@ -1703,84 +1795,97 @@
       <c r="J17" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="K17" s="11"/>
-      <c r="L17" s="11" t="n">
+      <c r="K17" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="L17" s="12" t="n">
         <f aca="false">SUM(B17:K17)</f>
-        <v>5</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="11" t="s">
         <v>73</v>
       </c>
-      <c r="B18" s="11"/>
-      <c r="C18" s="11"/>
-      <c r="D18" s="11"/>
-      <c r="E18" s="11"/>
+      <c r="B18" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="C18" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D18" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E18" s="11" t="n">
+        <v>0</v>
+      </c>
       <c r="F18" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="G18" s="11"/>
-      <c r="H18" s="11"/>
-      <c r="I18" s="11"/>
+        <v>3</v>
+      </c>
+      <c r="G18" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="I18" s="11" t="n">
+        <v>0</v>
+      </c>
       <c r="J18" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="K18" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="L18" s="11" t="n">
+      <c r="L18" s="12" t="n">
         <f aca="false">SUM(B18:K18)</f>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="s">
         <v>74</v>
       </c>
-      <c r="B19" s="12" t="n">
+      <c r="B19" s="13" t="n">
         <f aca="false">SUM(B4:B18)</f>
-        <v>112</v>
-      </c>
-      <c r="C19" s="12" t="n">
+        <v>130</v>
+      </c>
+      <c r="C19" s="13" t="n">
         <f aca="false">SUM(C4:C18)</f>
-        <v>107</v>
-      </c>
-      <c r="D19" s="12" t="n">
+        <v>134</v>
+      </c>
+      <c r="D19" s="13" t="n">
         <f aca="false">SUM(D4:D18)</f>
-        <v>91</v>
-      </c>
-      <c r="E19" s="12" t="n">
+        <v>118</v>
+      </c>
+      <c r="E19" s="13" t="n">
         <f aca="false">SUM(E4:E18)</f>
-        <v>88</v>
-      </c>
-      <c r="F19" s="12" t="n">
+        <v>114</v>
+      </c>
+      <c r="F19" s="13" t="n">
         <f aca="false">SUM(F4:F18)</f>
-        <v>114</v>
-      </c>
-      <c r="G19" s="12" t="n">
+        <v>136</v>
+      </c>
+      <c r="G19" s="13" t="n">
         <f aca="false">SUM(G4:G18)</f>
-        <v>150</v>
-      </c>
-      <c r="H19" s="12" t="n">
+        <v>177</v>
+      </c>
+      <c r="H19" s="13" t="n">
         <f aca="false">SUM(H4:H18)</f>
-        <v>136</v>
-      </c>
-      <c r="I19" s="12" t="n">
+        <v>163</v>
+      </c>
+      <c r="I19" s="13" t="n">
         <f aca="false">SUM(I4:I18)</f>
         <v>30</v>
       </c>
-      <c r="J19" s="12" t="n">
+      <c r="J19" s="13" t="n">
         <f aca="false">SUM(J4:J18)</f>
-        <v>112</v>
-      </c>
-      <c r="K19" s="12" t="n">
+        <v>145</v>
+      </c>
+      <c r="K19" s="13" t="n">
         <f aca="false">SUM(K4:K18)</f>
-        <v>139</v>
-      </c>
-      <c r="L19" s="12" t="n">
+        <v>154</v>
+      </c>
+      <c r="L19" s="13" t="n">
         <f aca="false">SUM(L4:L18)</f>
-        <v>1079</v>
+        <v>1301</v>
       </c>
     </row>
   </sheetData>
@@ -1802,8 +1907,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L28"/>
-  <sheetFormatPr defaultColWidth="8.66796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:L29"/>
+  <sheetFormatPr defaultColWidth="8.66796875" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="2" style="0" width="14"/>
@@ -1825,7 +1930,7 @@
       <c r="K1" s="10"/>
       <c r="L1" s="10"/>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
         <v>76</v>
       </c>
@@ -1863,825 +1968,879 @@
         <v>59</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="11" t="s">
+    <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="14" t="s">
         <v>77</v>
       </c>
-      <c r="B4" s="11" t="n">
+      <c r="B4" s="14" t="n">
+        <f aca="false">25+2</f>
+        <v>27</v>
+      </c>
+      <c r="C4" s="14" t="n">
+        <f aca="false">24+2</f>
+        <v>26</v>
+      </c>
+      <c r="D4" s="14" t="n">
+        <f aca="false">20+4</f>
+        <v>24</v>
+      </c>
+      <c r="E4" s="14" t="n">
+        <f aca="false">18+4</f>
+        <v>22</v>
+      </c>
+      <c r="F4" s="14" t="n">
+        <f aca="false">15+5</f>
+        <v>20</v>
+      </c>
+      <c r="G4" s="14" t="n">
+        <f aca="false">46+6</f>
+        <v>52</v>
+      </c>
+      <c r="H4" s="14" t="n">
+        <f aca="false">40+5</f>
+        <v>45</v>
+      </c>
+      <c r="I4" s="14"/>
+      <c r="J4" s="14" t="n">
+        <f aca="false">19+1</f>
+        <v>20</v>
+      </c>
+      <c r="K4" s="14" t="n">
+        <v>46</v>
+      </c>
+      <c r="L4" s="14" t="n">
+        <f aca="false">SUM(B4:K4)</f>
+        <v>282</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="14" t="s">
+        <v>78</v>
+      </c>
+      <c r="B5" s="14" t="n">
+        <v>19</v>
+      </c>
+      <c r="C5" s="14" t="n">
+        <v>20</v>
+      </c>
+      <c r="D5" s="14" t="n">
+        <v>7</v>
+      </c>
+      <c r="E5" s="14" t="n">
+        <v>19</v>
+      </c>
+      <c r="F5" s="14" t="n">
+        <v>34</v>
+      </c>
+      <c r="G5" s="14" t="n">
         <v>25</v>
       </c>
-      <c r="C4" s="11" t="n">
-        <v>24</v>
-      </c>
-      <c r="D4" s="11" t="n">
-        <v>20</v>
-      </c>
-      <c r="E4" s="11" t="n">
+      <c r="H5" s="14" t="n">
+        <v>21</v>
+      </c>
+      <c r="I5" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="J5" s="14" t="n">
+        <v>30</v>
+      </c>
+      <c r="K5" s="14" t="n">
         <v>18</v>
       </c>
-      <c r="F4" s="11" t="n">
-        <v>15</v>
-      </c>
-      <c r="G4" s="11" t="n">
-        <v>46</v>
-      </c>
-      <c r="H4" s="11" t="n">
-        <v>40</v>
-      </c>
-      <c r="I4" s="11"/>
-      <c r="J4" s="11" t="n">
-        <v>19</v>
-      </c>
-      <c r="K4" s="11" t="n">
-        <v>46</v>
-      </c>
-      <c r="L4" s="11" t="n">
-        <f aca="false">SUM(B4:K4)</f>
-        <v>253</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="11" t="s">
-        <v>78</v>
-      </c>
-      <c r="B5" s="11" t="n">
-        <v>19</v>
-      </c>
-      <c r="C5" s="11" t="n">
-        <v>20</v>
-      </c>
-      <c r="D5" s="11" t="n">
-        <v>7</v>
-      </c>
-      <c r="E5" s="11" t="n">
-        <v>19</v>
-      </c>
-      <c r="F5" s="11" t="n">
-        <v>34</v>
-      </c>
-      <c r="G5" s="11" t="n">
-        <v>25</v>
-      </c>
-      <c r="H5" s="11" t="n">
-        <v>21</v>
-      </c>
-      <c r="I5" s="11" t="n">
-        <v>6</v>
-      </c>
-      <c r="J5" s="11" t="n">
-        <v>30</v>
-      </c>
-      <c r="K5" s="11" t="n">
-        <v>18</v>
-      </c>
-      <c r="L5" s="11" t="n">
+      <c r="L5" s="14" t="n">
         <f aca="false">SUM(B5:K5)</f>
         <v>199</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="11" t="s">
+    <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="14" t="s">
         <v>79</v>
       </c>
-      <c r="B6" s="11" t="n">
+      <c r="B6" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="C6" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="D6" s="11" t="n">
+      <c r="C6" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="E6" s="11" t="n">
+      <c r="E6" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="F6" s="11" t="n">
+      <c r="F6" s="14" t="n">
         <v>17</v>
       </c>
-      <c r="G6" s="11" t="n">
+      <c r="G6" s="14" t="n">
         <v>26</v>
       </c>
-      <c r="H6" s="11" t="n">
+      <c r="H6" s="14" t="n">
         <v>20</v>
       </c>
-      <c r="I6" s="11" t="n">
+      <c r="I6" s="14" t="n">
         <v>9</v>
       </c>
-      <c r="J6" s="11" t="n">
+      <c r="J6" s="14" t="n">
         <v>28</v>
       </c>
-      <c r="K6" s="11" t="n">
+      <c r="K6" s="14" t="n">
         <v>28</v>
       </c>
-      <c r="L6" s="11" t="n">
+      <c r="L6" s="14" t="n">
         <f aca="false">SUM(B6:K6)</f>
         <v>142</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="11" t="s">
+    <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="14" t="s">
         <v>80</v>
       </c>
-      <c r="B7" s="11" t="n">
+      <c r="B7" s="14" t="n">
         <v>14</v>
       </c>
-      <c r="C7" s="11" t="n">
+      <c r="C7" s="14" t="n">
         <v>14</v>
       </c>
-      <c r="D7" s="11" t="n">
+      <c r="D7" s="14" t="n">
         <v>19</v>
       </c>
-      <c r="E7" s="11" t="n">
+      <c r="E7" s="14" t="n">
         <v>9</v>
       </c>
-      <c r="F7" s="11" t="n">
+      <c r="F7" s="14" t="n">
         <v>9</v>
       </c>
-      <c r="G7" s="11" t="n">
+      <c r="G7" s="14" t="n">
         <v>8</v>
       </c>
-      <c r="H7" s="11" t="n">
+      <c r="H7" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="I7" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="J7" s="11" t="n">
+      <c r="I7" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="J7" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="K7" s="11" t="n">
+      <c r="K7" s="14" t="n">
         <v>15</v>
       </c>
-      <c r="L7" s="11" t="n">
+      <c r="L7" s="14" t="n">
         <f aca="false">SUM(B7:K7)</f>
         <v>99</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="11" t="s">
+    <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="14" t="s">
         <v>81</v>
       </c>
-      <c r="B8" s="11" t="n">
+      <c r="B8" s="14" t="n">
         <v>10</v>
       </c>
-      <c r="C8" s="11" t="n">
+      <c r="C8" s="14" t="n">
         <v>10</v>
       </c>
-      <c r="D8" s="11" t="n">
+      <c r="D8" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="E8" s="11" t="n">
+      <c r="E8" s="14" t="n">
         <v>10</v>
       </c>
-      <c r="F8" s="11" t="n">
+      <c r="F8" s="14" t="n">
         <v>6</v>
       </c>
-      <c r="G8" s="11" t="n">
+      <c r="G8" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="H8" s="11" t="n">
+      <c r="H8" s="14" t="n">
         <v>10</v>
       </c>
-      <c r="I8" s="11" t="n">
+      <c r="I8" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="J8" s="11" t="n">
+      <c r="J8" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="K8" s="11" t="n">
+      <c r="K8" s="14" t="n">
         <v>8</v>
       </c>
-      <c r="L8" s="11" t="n">
+      <c r="L8" s="14" t="n">
         <f aca="false">SUM(B8:K8)</f>
         <v>71</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="11" t="s">
+    <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="14" t="s">
         <v>82</v>
       </c>
-      <c r="B9" s="11" t="n">
+      <c r="B9" s="14" t="n">
         <v>7</v>
       </c>
-      <c r="C9" s="11" t="n">
+      <c r="C9" s="14" t="n">
         <v>7</v>
       </c>
-      <c r="D9" s="11" t="n">
+      <c r="D9" s="14" t="n">
         <v>16</v>
       </c>
-      <c r="E9" s="11" t="n">
+      <c r="E9" s="14" t="n">
         <v>13</v>
       </c>
-      <c r="F9" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="G9" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="H9" s="11" t="n">
+      <c r="F9" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="G9" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="H9" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="I9" s="11"/>
-      <c r="J9" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="K9" s="11" t="n">
+      <c r="I9" s="14"/>
+      <c r="J9" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="K9" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="L9" s="11" t="n">
+      <c r="L9" s="14" t="n">
         <f aca="false">SUM(B9:K9)</f>
         <v>57</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="11" t="s">
+    <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="14" t="s">
         <v>83</v>
       </c>
-      <c r="B10" s="11" t="n">
+      <c r="B10" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="C10" s="11" t="n">
+      <c r="C10" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="D10" s="11" t="n">
+      <c r="D10" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="E10" s="11" t="n">
+      <c r="E10" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="F10" s="11" t="n">
+      <c r="F10" s="14" t="n">
         <v>7</v>
       </c>
-      <c r="G10" s="11" t="n">
+      <c r="G10" s="14" t="n">
         <v>6</v>
       </c>
-      <c r="H10" s="11" t="n">
+      <c r="H10" s="14" t="n">
         <v>6</v>
       </c>
-      <c r="I10" s="11" t="n">
+      <c r="I10" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="J10" s="11" t="n">
+      <c r="J10" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="K10" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="L10" s="11" t="n">
+      <c r="K10" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="L10" s="14" t="n">
         <f aca="false">SUM(B10:K10)</f>
         <v>44</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="11" t="s">
+    <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="14" t="s">
         <v>84</v>
       </c>
-      <c r="B11" s="11" t="n">
+      <c r="B11" s="14" t="n">
         <v>12</v>
       </c>
-      <c r="C11" s="11" t="n">
+      <c r="C11" s="14" t="n">
         <v>8</v>
       </c>
-      <c r="D11" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="E11" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="F11" s="11" t="n">
+      <c r="D11" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="E11" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="F11" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="G11" s="11" t="n">
+      <c r="G11" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="H11" s="11" t="n">
+      <c r="H11" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="I11" s="11"/>
-      <c r="J11" s="11" t="n">
+      <c r="I11" s="14"/>
+      <c r="J11" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="K11" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="L11" s="11" t="n">
+      <c r="K11" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="L11" s="14" t="n">
         <f aca="false">SUM(B11:K11)</f>
         <v>39</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="11" t="s">
+    <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="14" t="s">
         <v>85</v>
       </c>
-      <c r="B12" s="11" t="n">
+      <c r="B12" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="C12" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="D12" s="11" t="n">
+      <c r="C12" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="D12" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="E12" s="11" t="n">
+      <c r="E12" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="F12" s="11" t="n">
+      <c r="F12" s="14" t="n">
         <v>7</v>
       </c>
-      <c r="G12" s="11" t="n">
+      <c r="G12" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="H12" s="11" t="n">
+      <c r="H12" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="I12" s="11" t="n">
+      <c r="I12" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="J12" s="11" t="n">
+      <c r="J12" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="K12" s="11"/>
-      <c r="L12" s="11" t="n">
+      <c r="K12" s="14"/>
+      <c r="L12" s="14" t="n">
         <f aca="false">SUM(B12:K12)</f>
         <v>36</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="11" t="s">
+    <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="14" t="s">
         <v>86</v>
       </c>
-      <c r="B13" s="11"/>
-      <c r="C13" s="11" t="n">
+      <c r="B13" s="14"/>
+      <c r="C13" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="D13" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="E13" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="F13" s="11" t="n">
+      <c r="D13" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="F13" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="G13" s="11" t="n">
+      <c r="G13" s="14" t="n">
         <v>7</v>
       </c>
-      <c r="H13" s="11" t="n">
+      <c r="H13" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="I13" s="11"/>
-      <c r="J13" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="K13" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="L13" s="11" t="n">
+      <c r="I13" s="14"/>
+      <c r="J13" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="K13" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="L13" s="14" t="n">
         <f aca="false">SUM(B13:K13)</f>
         <v>22</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="11" t="s">
+    <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="14" t="s">
         <v>87</v>
       </c>
-      <c r="B14" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="C14" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="D14" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="E14" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="F14" s="11"/>
-      <c r="G14" s="11" t="n">
+      <c r="B14" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="C14" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="F14" s="14"/>
+      <c r="G14" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="H14" s="11" t="n">
+      <c r="H14" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="I14" s="11"/>
-      <c r="J14" s="11" t="n">
+      <c r="I14" s="14"/>
+      <c r="J14" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="K14" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="L14" s="11" t="n">
+      <c r="K14" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="L14" s="14" t="n">
         <f aca="false">SUM(B14:K14)</f>
         <v>19</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="11" t="s">
+    <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="14" t="s">
         <v>88</v>
       </c>
-      <c r="B15" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="C15" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="D15" s="11"/>
-      <c r="E15" s="11" t="n">
+      <c r="B15" s="14" t="n">
+        <f aca="false">1+2</f>
         <v>3</v>
       </c>
-      <c r="F15" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="G15" s="11" t="n">
-        <v>5</v>
-      </c>
-      <c r="H15" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="I15" s="11"/>
-      <c r="J15" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="K15" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="L15" s="11" t="n">
+      <c r="C15" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="D15" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="E15" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="F15" s="14" t="n">
+        <f aca="false">1+1</f>
+        <v>2</v>
+      </c>
+      <c r="G15" s="14" t="n">
+        <f aca="false">5+2</f>
+        <v>7</v>
+      </c>
+      <c r="H15" s="14" t="n">
+        <f aca="false">1+3</f>
+        <v>4</v>
+      </c>
+      <c r="I15" s="14"/>
+      <c r="J15" s="14" t="n">
+        <f aca="false">1+1</f>
+        <v>2</v>
+      </c>
+      <c r="K15" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="L15" s="14" t="n">
         <f aca="false">SUM(B15:K15)</f>
-        <v>16</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="11" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="14" t="s">
         <v>89</v>
       </c>
-      <c r="B16" s="11" t="n">
+      <c r="B16" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="C16" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="D16" s="11" t="n">
+      <c r="C16" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="D16" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="E16" s="11"/>
-      <c r="F16" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="G16" s="11"/>
-      <c r="H16" s="11" t="n">
+      <c r="E16" s="14"/>
+      <c r="F16" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="G16" s="14"/>
+      <c r="H16" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="I16" s="11"/>
-      <c r="J16" s="11" t="n">
+      <c r="I16" s="14"/>
+      <c r="J16" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="K16" s="11"/>
-      <c r="L16" s="11" t="n">
+      <c r="K16" s="14"/>
+      <c r="L16" s="14" t="n">
         <f aca="false">SUM(B16:K16)</f>
         <v>16</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="11" t="s">
+    <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="14" t="s">
         <v>90</v>
       </c>
-      <c r="B17" s="11"/>
-      <c r="C17" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="D17" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="E17" s="11"/>
-      <c r="F17" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="G17" s="11"/>
-      <c r="H17" s="11" t="n">
+      <c r="B17" s="14"/>
+      <c r="C17" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="D17" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="E17" s="14"/>
+      <c r="F17" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="G17" s="14"/>
+      <c r="H17" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="I17" s="11"/>
-      <c r="J17" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="K17" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="L17" s="11" t="n">
+      <c r="I17" s="14"/>
+      <c r="J17" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="K17" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="L17" s="14" t="n">
         <f aca="false">SUM(B17:K17)</f>
         <v>11</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="11" t="s">
+    <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="14" t="s">
         <v>91</v>
       </c>
-      <c r="B18" s="11"/>
-      <c r="C18" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="D18" s="11"/>
-      <c r="E18" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="F18" s="11" t="n">
+      <c r="B18" s="14"/>
+      <c r="C18" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="D18" s="14"/>
+      <c r="E18" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="F18" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="G18" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="H18" s="11"/>
-      <c r="I18" s="11"/>
-      <c r="J18" s="11"/>
-      <c r="K18" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="L18" s="11" t="n">
+      <c r="G18" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="H18" s="14"/>
+      <c r="I18" s="14"/>
+      <c r="J18" s="14"/>
+      <c r="K18" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="L18" s="14" t="n">
         <f aca="false">SUM(B18:K18)</f>
         <v>10</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="11" t="s">
+    <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="14" t="s">
         <v>92</v>
       </c>
-      <c r="B19" s="11" t="n">
+      <c r="B19" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="C19" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="D19" s="11"/>
-      <c r="E19" s="11"/>
-      <c r="F19" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="G19" s="11"/>
-      <c r="H19" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="I19" s="11"/>
-      <c r="J19" s="11"/>
-      <c r="K19" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="L19" s="11" t="n">
+      <c r="C19" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="D19" s="14"/>
+      <c r="E19" s="14"/>
+      <c r="F19" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="G19" s="14"/>
+      <c r="H19" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="I19" s="14"/>
+      <c r="J19" s="14"/>
+      <c r="K19" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="L19" s="14" t="n">
         <f aca="false">SUM(B19:K19)</f>
         <v>10</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="11" t="s">
+    <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="14" t="s">
         <v>93</v>
       </c>
-      <c r="B20" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="C20" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="D20" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="E20" s="11"/>
-      <c r="F20" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="G20" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="H20" s="11"/>
-      <c r="I20" s="11"/>
-      <c r="J20" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="K20" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="L20" s="11" t="n">
+      <c r="B20" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="C20" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="D20" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="E20" s="14"/>
+      <c r="F20" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="G20" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="H20" s="14"/>
+      <c r="I20" s="14"/>
+      <c r="J20" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="K20" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="L20" s="14" t="n">
         <f aca="false">SUM(B20:K20)</f>
         <v>8</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="11" t="s">
+    <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="14" t="s">
         <v>94</v>
       </c>
-      <c r="B21" s="11"/>
-      <c r="C21" s="11"/>
-      <c r="D21" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="E21" s="11"/>
-      <c r="F21" s="11"/>
-      <c r="G21" s="11" t="n">
+      <c r="B21" s="14"/>
+      <c r="C21" s="14"/>
+      <c r="D21" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="E21" s="14"/>
+      <c r="F21" s="14"/>
+      <c r="G21" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="H21" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="I21" s="11"/>
-      <c r="J21" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="K21" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="L21" s="11" t="n">
+      <c r="H21" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="I21" s="14"/>
+      <c r="J21" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="K21" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="L21" s="14" t="n">
         <f aca="false">SUM(B21:K21)</f>
         <v>7</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="11" t="s">
+    <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="14" t="s">
         <v>95</v>
       </c>
-      <c r="B22" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="C22" s="11"/>
-      <c r="D22" s="11"/>
-      <c r="E22" s="11"/>
-      <c r="F22" s="11"/>
-      <c r="G22" s="11"/>
-      <c r="H22" s="11" t="n">
+      <c r="B22" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="C22" s="14"/>
+      <c r="D22" s="14"/>
+      <c r="E22" s="14"/>
+      <c r="F22" s="14"/>
+      <c r="G22" s="14"/>
+      <c r="H22" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="I22" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="J22" s="11"/>
-      <c r="K22" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="L22" s="11" t="n">
+      <c r="I22" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="J22" s="14"/>
+      <c r="K22" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="L22" s="14" t="n">
         <f aca="false">SUM(B22:K22)</f>
         <v>6</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="11" t="s">
+    <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="14" t="s">
         <v>96</v>
       </c>
-      <c r="B23" s="11"/>
-      <c r="C23" s="11"/>
-      <c r="D23" s="11"/>
-      <c r="E23" s="11"/>
-      <c r="F23" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="G23" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="H23" s="11"/>
-      <c r="I23" s="11"/>
-      <c r="J23" s="11"/>
-      <c r="K23" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="L23" s="11" t="n">
+      <c r="B23" s="14"/>
+      <c r="C23" s="14"/>
+      <c r="D23" s="14"/>
+      <c r="E23" s="14"/>
+      <c r="F23" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="G23" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="H23" s="14"/>
+      <c r="I23" s="14"/>
+      <c r="J23" s="14"/>
+      <c r="K23" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="L23" s="14" t="n">
         <f aca="false">SUM(B23:K23)</f>
         <v>4</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="11" t="s">
+    <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="14" t="s">
         <v>97</v>
       </c>
-      <c r="B24" s="11"/>
-      <c r="C24" s="11"/>
-      <c r="D24" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="E24" s="11"/>
-      <c r="F24" s="11"/>
-      <c r="G24" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="H24" s="11"/>
-      <c r="I24" s="11"/>
-      <c r="J24" s="11"/>
-      <c r="K24" s="11"/>
-      <c r="L24" s="11" t="n">
+      <c r="B24" s="14"/>
+      <c r="C24" s="14"/>
+      <c r="D24" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="E24" s="14"/>
+      <c r="F24" s="14"/>
+      <c r="G24" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="H24" s="14"/>
+      <c r="I24" s="14"/>
+      <c r="J24" s="14"/>
+      <c r="K24" s="14"/>
+      <c r="L24" s="14" t="n">
         <f aca="false">SUM(B24:K24)</f>
         <v>3</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="11" t="s">
+    <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="14" t="s">
         <v>98</v>
       </c>
-      <c r="B25" s="11"/>
-      <c r="C25" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="D25" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="E25" s="11"/>
-      <c r="F25" s="11"/>
-      <c r="G25" s="11"/>
-      <c r="H25" s="11"/>
-      <c r="I25" s="11"/>
-      <c r="J25" s="11"/>
-      <c r="K25" s="11"/>
-      <c r="L25" s="11" t="n">
+      <c r="B25" s="14"/>
+      <c r="C25" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="D25" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="E25" s="14"/>
+      <c r="F25" s="14"/>
+      <c r="G25" s="14"/>
+      <c r="H25" s="14"/>
+      <c r="I25" s="14"/>
+      <c r="J25" s="14"/>
+      <c r="K25" s="14"/>
+      <c r="L25" s="14" t="n">
         <f aca="false">SUM(B25:K25)</f>
         <v>3</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="11" t="s">
+    <row r="26" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="14" t="s">
         <v>99</v>
       </c>
-      <c r="B26" s="11"/>
-      <c r="C26" s="11"/>
-      <c r="D26" s="11"/>
-      <c r="E26" s="11"/>
-      <c r="F26" s="11"/>
-      <c r="G26" s="11"/>
-      <c r="H26" s="11"/>
-      <c r="I26" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="J26" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="K26" s="11"/>
-      <c r="L26" s="11" t="n">
+      <c r="B26" s="14"/>
+      <c r="C26" s="14"/>
+      <c r="D26" s="14"/>
+      <c r="E26" s="14"/>
+      <c r="F26" s="14"/>
+      <c r="G26" s="14"/>
+      <c r="H26" s="14"/>
+      <c r="I26" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="J26" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="K26" s="14"/>
+      <c r="L26" s="14" t="n">
         <f aca="false">SUM(B26:K26)</f>
         <v>2</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="11" t="s">
+    <row r="27" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="14" t="s">
         <v>100</v>
       </c>
-      <c r="B27" s="11"/>
-      <c r="C27" s="11"/>
-      <c r="D27" s="11"/>
-      <c r="E27" s="11"/>
-      <c r="F27" s="11"/>
-      <c r="G27" s="11"/>
-      <c r="H27" s="11"/>
-      <c r="I27" s="11"/>
-      <c r="J27" s="11"/>
-      <c r="K27" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="L27" s="11" t="n">
+      <c r="B27" s="14"/>
+      <c r="C27" s="14"/>
+      <c r="D27" s="14"/>
+      <c r="E27" s="14"/>
+      <c r="F27" s="14"/>
+      <c r="G27" s="14"/>
+      <c r="H27" s="14"/>
+      <c r="I27" s="14"/>
+      <c r="J27" s="14"/>
+      <c r="K27" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="L27" s="14" t="n">
         <f aca="false">SUM(B27:K27)</f>
         <v>1</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="7" t="s">
+    <row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="14" t="s">
+        <v>101</v>
+      </c>
+      <c r="B28" s="14" t="n">
+        <v>14</v>
+      </c>
+      <c r="C28" s="14" t="n">
+        <v>27</v>
+      </c>
+      <c r="D28" s="14" t="n">
+        <v>27</v>
+      </c>
+      <c r="E28" s="14" t="n">
+        <v>26</v>
+      </c>
+      <c r="F28" s="14" t="n">
+        <v>22</v>
+      </c>
+      <c r="G28" s="14" t="n">
+        <v>27</v>
+      </c>
+      <c r="H28" s="14" t="n">
+        <v>27</v>
+      </c>
+      <c r="I28" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="J28" s="14" t="n">
+        <v>33</v>
+      </c>
+      <c r="K28" s="14" t="n">
+        <v>16</v>
+      </c>
+      <c r="L28" s="14" t="n">
+        <f aca="false">SUM(B28:K28)</f>
+        <v>219</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="7" t="s">
         <v>74</v>
       </c>
-      <c r="B28" s="7" t="n">
-        <f aca="false">SUM(B4:B27)</f>
-        <v>111</v>
-      </c>
-      <c r="C28" s="7" t="n">
-        <f aca="false">SUM(C4:C27)</f>
-        <v>107</v>
-      </c>
-      <c r="D28" s="7" t="n">
-        <f aca="false">SUM(D4:D27)</f>
-        <v>91</v>
-      </c>
-      <c r="E28" s="7" t="n">
-        <f aca="false">SUM(E4:E27)</f>
-        <v>88</v>
-      </c>
-      <c r="F28" s="7" t="n">
-        <f aca="false">SUM(F4:F27)</f>
-        <v>114</v>
-      </c>
-      <c r="G28" s="7" t="n">
-        <f aca="false">SUM(G4:G27)</f>
-        <v>150</v>
-      </c>
-      <c r="H28" s="7" t="n">
-        <f aca="false">SUM(H4:H27)</f>
+      <c r="B29" s="7" t="n">
+        <f aca="false">SUM(B4:B28)</f>
+        <v>129</v>
+      </c>
+      <c r="C29" s="7" t="n">
+        <f aca="false">SUM(C4:C28)</f>
         <v>136</v>
       </c>
-      <c r="I28" s="7" t="n">
-        <f aca="false">SUM(I4:I27)</f>
+      <c r="D29" s="7" t="n">
+        <f aca="false">SUM(D4:D28)</f>
+        <v>124</v>
+      </c>
+      <c r="E29" s="7" t="n">
+        <f aca="false">SUM(E4:E28)</f>
+        <v>118</v>
+      </c>
+      <c r="F29" s="7" t="n">
+        <f aca="false">SUM(F4:F28)</f>
+        <v>142</v>
+      </c>
+      <c r="G29" s="7" t="n">
+        <f aca="false">SUM(G4:G28)</f>
+        <v>185</v>
+      </c>
+      <c r="H29" s="7" t="n">
+        <f aca="false">SUM(H4:H28)</f>
+        <v>171</v>
+      </c>
+      <c r="I29" s="7" t="n">
+        <f aca="false">SUM(I4:I28)</f>
         <v>30</v>
       </c>
-      <c r="J28" s="7" t="n">
-        <f aca="false">SUM(J4:J27)</f>
-        <v>112</v>
-      </c>
-      <c r="K28" s="7" t="n">
-        <f aca="false">SUM(K4:K27)</f>
-        <v>139</v>
-      </c>
-      <c r="L28" s="7" t="n">
-        <f aca="false">SUM(L4:L27)</f>
-        <v>1078</v>
+      <c r="J29" s="7" t="n">
+        <f aca="false">SUM(J4:J28)</f>
+        <v>147</v>
+      </c>
+      <c r="K29" s="7" t="n">
+        <f aca="false">SUM(K4:K28)</f>
+        <v>155</v>
+      </c>
+      <c r="L29" s="7" t="n">
+        <f aca="false">SUM(L4:L28)</f>
+        <v>1337</v>
       </c>
     </row>
   </sheetData>
@@ -2703,8 +2862,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L28"/>
-  <sheetFormatPr defaultColWidth="8.66796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:L29"/>
+  <sheetFormatPr defaultColWidth="8.66796875" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="2" style="0" width="14"/>
@@ -2712,7 +2871,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="10" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B1" s="10"/>
       <c r="C1" s="10"/>
@@ -2726,7 +2885,7 @@
       <c r="K1" s="10"/>
       <c r="L1" s="10"/>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
         <v>76</v>
       </c>
@@ -2764,837 +2923,890 @@
         <v>59</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="11" t="s">
+    <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="14" t="s">
         <v>89</v>
       </c>
-      <c r="B4" s="11" t="n">
-        <v>179</v>
-      </c>
-      <c r="C4" s="11" t="n">
-        <v>283.5</v>
-      </c>
-      <c r="D4" s="11" t="n">
-        <v>132.75</v>
-      </c>
-      <c r="E4" s="11" t="n">
-        <v>160</v>
-      </c>
-      <c r="F4" s="11" t="n">
-        <v>195</v>
-      </c>
-      <c r="G4" s="11" t="n">
-        <v>224.75</v>
-      </c>
-      <c r="H4" s="11" t="n">
-        <v>202.65</v>
-      </c>
-      <c r="I4" s="11" t="n">
+      <c r="B4" s="14" t="n">
+        <f aca="false">179+21</f>
+        <v>200</v>
+      </c>
+      <c r="C4" s="14" t="n">
+        <f aca="false">283.5+4</f>
+        <v>287.5</v>
+      </c>
+      <c r="D4" s="14" t="n">
+        <f aca="false">132.75+33</f>
+        <v>165.75</v>
+      </c>
+      <c r="E4" s="14" t="n">
+        <f aca="false">160+13</f>
+        <v>173</v>
+      </c>
+      <c r="F4" s="14" t="n">
+        <f aca="false">195+47</f>
+        <v>242</v>
+      </c>
+      <c r="G4" s="14" t="n">
+        <f aca="false">224.75+19</f>
+        <v>243.75</v>
+      </c>
+      <c r="H4" s="14" t="n">
+        <f aca="false">202.65+23</f>
+        <v>225.65</v>
+      </c>
+      <c r="I4" s="14" t="n">
         <v>276.75</v>
       </c>
-      <c r="J4" s="11" t="n">
-        <v>298.25</v>
-      </c>
-      <c r="K4" s="11" t="n">
+      <c r="J4" s="14" t="n">
+        <f aca="false">298.25+1</f>
+        <v>299.25</v>
+      </c>
+      <c r="K4" s="14" t="n">
         <v>59.25</v>
       </c>
-      <c r="L4" s="11" t="n">
+      <c r="L4" s="14" t="n">
         <f aca="false">SUM(B4:K4)</f>
-        <v>2011.9</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="11" t="s">
+        <v>2172.9</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="14" t="s">
         <v>79</v>
       </c>
-      <c r="B5" s="11" t="n">
+      <c r="B5" s="14" t="n">
         <v>13</v>
       </c>
-      <c r="C5" s="11" t="n">
+      <c r="C5" s="14" t="n">
         <v>6</v>
       </c>
-      <c r="D5" s="11" t="n">
+      <c r="D5" s="14" t="n">
         <v>34.5</v>
       </c>
-      <c r="E5" s="11" t="n">
+      <c r="E5" s="14" t="n">
         <v>36</v>
       </c>
-      <c r="F5" s="11" t="n">
+      <c r="F5" s="14" t="n">
         <v>82</v>
       </c>
-      <c r="G5" s="11" t="n">
+      <c r="G5" s="14" t="n">
         <v>129.75</v>
       </c>
-      <c r="H5" s="11" t="n">
+      <c r="H5" s="14" t="n">
         <v>94.5</v>
       </c>
-      <c r="I5" s="11" t="n">
+      <c r="I5" s="14" t="n">
         <v>74.5</v>
       </c>
-      <c r="J5" s="11" t="n">
+      <c r="J5" s="14" t="n">
         <v>137</v>
       </c>
-      <c r="K5" s="11" t="n">
+      <c r="K5" s="14" t="n">
         <v>119.5</v>
       </c>
-      <c r="L5" s="11" t="n">
+      <c r="L5" s="14" t="n">
         <f aca="false">SUM(B5:K5)</f>
         <v>726.75</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="11" t="s">
+    <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="B6" s="11" t="n">
+      <c r="B6" s="14" t="n">
         <v>149.75</v>
       </c>
-      <c r="C6" s="11" t="n">
+      <c r="C6" s="14" t="n">
         <v>25.5</v>
       </c>
-      <c r="D6" s="11" t="n">
+      <c r="D6" s="14" t="n">
         <v>53.25</v>
       </c>
-      <c r="E6" s="11" t="n">
+      <c r="E6" s="14" t="n">
         <v>60.8</v>
       </c>
-      <c r="F6" s="11" t="n">
+      <c r="F6" s="14" t="n">
         <v>96.25</v>
       </c>
-      <c r="G6" s="11" t="n">
+      <c r="G6" s="14" t="n">
         <v>99</v>
       </c>
-      <c r="H6" s="11" t="n">
+      <c r="H6" s="14" t="n">
         <v>71.65</v>
       </c>
-      <c r="I6" s="11" t="n">
+      <c r="I6" s="14" t="n">
         <v>17.25</v>
       </c>
-      <c r="J6" s="11" t="n">
+      <c r="J6" s="14" t="n">
         <v>96.75</v>
       </c>
-      <c r="K6" s="11" t="n">
+      <c r="K6" s="14" t="n">
         <v>29.25</v>
       </c>
-      <c r="L6" s="11" t="n">
+      <c r="L6" s="14" t="n">
         <f aca="false">SUM(B6:K6)</f>
         <v>699.45</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="11" t="s">
+    <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="14" t="s">
         <v>77</v>
       </c>
-      <c r="B7" s="11" t="n">
+      <c r="B7" s="14" t="n">
         <v>27.5</v>
       </c>
-      <c r="C7" s="11" t="n">
+      <c r="C7" s="14" t="n">
         <v>62.25</v>
       </c>
-      <c r="D7" s="11" t="n">
+      <c r="D7" s="14" t="n">
         <v>102.5</v>
       </c>
-      <c r="E7" s="11" t="n">
+      <c r="E7" s="14" t="n">
         <v>60</v>
       </c>
-      <c r="F7" s="11" t="n">
+      <c r="F7" s="14" t="n">
         <v>26.75</v>
       </c>
-      <c r="G7" s="11" t="n">
+      <c r="G7" s="14" t="n">
         <v>70.55</v>
       </c>
-      <c r="H7" s="11" t="n">
+      <c r="H7" s="14" t="n">
         <v>84.85</v>
       </c>
-      <c r="I7" s="11" t="n">
+      <c r="I7" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="J7" s="11" t="n">
+      <c r="J7" s="14" t="n">
         <v>39.75</v>
       </c>
-      <c r="K7" s="11" t="n">
+      <c r="K7" s="14" t="n">
         <v>95.5</v>
       </c>
-      <c r="L7" s="11" t="n">
+      <c r="L7" s="14" t="n">
         <f aca="false">SUM(B7:K7)</f>
         <v>572.65</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="11" t="s">
+    <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="14" t="s">
         <v>81</v>
       </c>
-      <c r="B8" s="11" t="n">
+      <c r="B8" s="14" t="n">
         <v>89</v>
       </c>
-      <c r="C8" s="11" t="n">
+      <c r="C8" s="14" t="n">
         <v>65.5</v>
       </c>
-      <c r="D8" s="11" t="n">
+      <c r="D8" s="14" t="n">
         <v>28</v>
       </c>
-      <c r="E8" s="11" t="n">
+      <c r="E8" s="14" t="n">
         <v>66</v>
       </c>
-      <c r="F8" s="11" t="n">
+      <c r="F8" s="14" t="n">
         <v>19.75</v>
       </c>
-      <c r="G8" s="11" t="n">
+      <c r="G8" s="14" t="n">
         <v>9.75</v>
       </c>
-      <c r="H8" s="11" t="n">
+      <c r="H8" s="14" t="n">
         <v>32.25</v>
       </c>
-      <c r="I8" s="11" t="n">
+      <c r="I8" s="14" t="n">
         <v>11.5</v>
       </c>
-      <c r="J8" s="11" t="n">
+      <c r="J8" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="K8" s="11" t="n">
+      <c r="K8" s="14" t="n">
         <v>23.5</v>
       </c>
-      <c r="L8" s="11" t="n">
+      <c r="L8" s="14" t="n">
         <f aca="false">SUM(B8:K8)</f>
         <v>350.25</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="11" t="s">
+    <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="14" t="s">
         <v>82</v>
       </c>
-      <c r="B9" s="11" t="n">
+      <c r="B9" s="14" t="n">
         <v>29.25</v>
       </c>
-      <c r="C9" s="11" t="n">
+      <c r="C9" s="14" t="n">
         <v>43.5</v>
       </c>
-      <c r="D9" s="11" t="n">
+      <c r="D9" s="14" t="n">
         <v>71.5</v>
       </c>
-      <c r="E9" s="11" t="n">
+      <c r="E9" s="14" t="n">
         <v>84</v>
       </c>
-      <c r="F9" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="G9" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="H9" s="11" t="n">
+      <c r="F9" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="G9" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="H9" s="14" t="n">
         <v>34</v>
       </c>
-      <c r="I9" s="11"/>
-      <c r="J9" s="11" t="n">
+      <c r="I9" s="14"/>
+      <c r="J9" s="14" t="n">
         <v>21.25</v>
       </c>
-      <c r="K9" s="11" t="n">
+      <c r="K9" s="14" t="n">
         <v>12</v>
       </c>
-      <c r="L9" s="11" t="n">
+      <c r="L9" s="14" t="n">
         <f aca="false">SUM(B9:K9)</f>
         <v>297.5</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="11" t="s">
+    <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="14" t="s">
         <v>83</v>
       </c>
-      <c r="B10" s="11" t="n">
+      <c r="B10" s="14" t="n">
         <v>16.75</v>
       </c>
-      <c r="C10" s="11" t="n">
+      <c r="C10" s="14" t="n">
         <v>8</v>
       </c>
-      <c r="D10" s="11" t="n">
+      <c r="D10" s="14" t="n">
         <v>38</v>
       </c>
-      <c r="E10" s="11" t="n">
+      <c r="E10" s="14" t="n">
         <v>40.5</v>
       </c>
-      <c r="F10" s="11" t="n">
+      <c r="F10" s="14" t="n">
         <v>37.5</v>
       </c>
-      <c r="G10" s="11" t="n">
+      <c r="G10" s="14" t="n">
         <v>32</v>
       </c>
-      <c r="H10" s="11" t="n">
+      <c r="H10" s="14" t="n">
         <v>34.5</v>
       </c>
-      <c r="I10" s="11" t="n">
+      <c r="I10" s="14" t="n">
         <v>6.5</v>
       </c>
-      <c r="J10" s="11" t="n">
+      <c r="J10" s="14" t="n">
         <v>29</v>
       </c>
-      <c r="K10" s="11" t="n">
+      <c r="K10" s="14" t="n">
         <v>2.5</v>
       </c>
-      <c r="L10" s="11" t="n">
+      <c r="L10" s="14" t="n">
         <f aca="false">SUM(B10:K10)</f>
         <v>245.25</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="11" t="s">
+    <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="14" t="s">
         <v>84</v>
       </c>
-      <c r="B11" s="11" t="n">
+      <c r="B11" s="14" t="n">
         <v>74</v>
       </c>
-      <c r="C11" s="11" t="n">
+      <c r="C11" s="14" t="n">
         <v>53.5</v>
       </c>
-      <c r="D11" s="11" t="n">
+      <c r="D11" s="14" t="n">
         <v>28.5</v>
       </c>
-      <c r="E11" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="F11" s="11" t="n">
+      <c r="E11" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="F11" s="14" t="n">
         <v>24.75</v>
       </c>
-      <c r="G11" s="11" t="n">
+      <c r="G11" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="H11" s="11" t="n">
+      <c r="H11" s="14" t="n">
         <v>21.5</v>
       </c>
-      <c r="I11" s="11"/>
-      <c r="J11" s="11" t="n">
+      <c r="I11" s="14"/>
+      <c r="J11" s="14" t="n">
         <v>21</v>
       </c>
-      <c r="K11" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="L11" s="11" t="n">
+      <c r="K11" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="L11" s="14" t="n">
         <f aca="false">SUM(B11:K11)</f>
         <v>230.25</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="11" t="s">
+    <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="14" t="s">
         <v>85</v>
       </c>
-      <c r="B12" s="11" t="n">
+      <c r="B12" s="14" t="n">
         <v>24.25</v>
       </c>
-      <c r="C12" s="11" t="n">
+      <c r="C12" s="14" t="n">
         <v>15</v>
       </c>
-      <c r="D12" s="11" t="n">
+      <c r="D12" s="14" t="n">
         <v>11.5</v>
       </c>
-      <c r="E12" s="11" t="n">
+      <c r="E12" s="14" t="n">
         <v>20.5</v>
       </c>
-      <c r="F12" s="11" t="n">
+      <c r="F12" s="14" t="n">
         <v>32.5</v>
       </c>
-      <c r="G12" s="11" t="n">
+      <c r="G12" s="14" t="n">
         <v>11</v>
       </c>
-      <c r="H12" s="11" t="n">
+      <c r="H12" s="14" t="n">
         <v>31</v>
       </c>
-      <c r="I12" s="11" t="n">
+      <c r="I12" s="14" t="n">
         <v>29.25</v>
       </c>
-      <c r="J12" s="11" t="n">
+      <c r="J12" s="14" t="n">
         <v>33.25</v>
       </c>
-      <c r="K12" s="11"/>
-      <c r="L12" s="11" t="n">
+      <c r="K12" s="14"/>
+      <c r="L12" s="14" t="n">
         <f aca="false">SUM(B12:K12)</f>
         <v>208.25</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="11" t="s">
+    <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="14" t="s">
         <v>80</v>
       </c>
-      <c r="B13" s="11" t="n">
+      <c r="B13" s="14" t="n">
         <v>9</v>
       </c>
-      <c r="C13" s="11" t="n">
+      <c r="C13" s="14" t="n">
         <v>13</v>
       </c>
-      <c r="D13" s="11" t="n">
+      <c r="D13" s="14" t="n">
         <v>18.25</v>
       </c>
-      <c r="E13" s="11" t="n">
+      <c r="E13" s="14" t="n">
         <v>17.5</v>
       </c>
-      <c r="F13" s="11" t="n">
+      <c r="F13" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="G13" s="11" t="n">
+      <c r="G13" s="14" t="n">
         <v>7.75</v>
       </c>
-      <c r="H13" s="11" t="n">
+      <c r="H13" s="14" t="n">
         <v>5.25</v>
       </c>
-      <c r="I13" s="11" t="n">
+      <c r="I13" s="14" t="n">
         <v>2.5</v>
       </c>
-      <c r="J13" s="11" t="n">
+      <c r="J13" s="14" t="n">
         <v>4.75</v>
       </c>
-      <c r="K13" s="11" t="n">
+      <c r="K13" s="14" t="n">
         <v>8.5</v>
       </c>
-      <c r="L13" s="11" t="n">
+      <c r="L13" s="14" t="n">
         <f aca="false">SUM(B13:K13)</f>
         <v>91.5</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="11" t="s">
+    <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="14" t="s">
         <v>91</v>
       </c>
-      <c r="B14" s="11"/>
-      <c r="C14" s="11" t="n">
+      <c r="B14" s="14"/>
+      <c r="C14" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="D14" s="11"/>
-      <c r="E14" s="11" t="n">
+      <c r="D14" s="14"/>
+      <c r="E14" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="F14" s="11" t="n">
+      <c r="F14" s="14" t="n">
         <v>48</v>
       </c>
-      <c r="G14" s="11" t="n">
+      <c r="G14" s="14" t="n">
         <v>10.5</v>
       </c>
-      <c r="H14" s="11"/>
-      <c r="I14" s="11"/>
-      <c r="J14" s="11"/>
-      <c r="K14" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="L14" s="11" t="n">
+      <c r="H14" s="14"/>
+      <c r="I14" s="14"/>
+      <c r="J14" s="14"/>
+      <c r="K14" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="L14" s="14" t="n">
         <f aca="false">SUM(B14:K14)</f>
         <v>68.5</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="11" t="s">
+    <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="14" t="s">
         <v>86</v>
       </c>
-      <c r="B15" s="11"/>
-      <c r="C15" s="11" t="n">
+      <c r="B15" s="14"/>
+      <c r="C15" s="14" t="n">
         <v>14.5</v>
       </c>
-      <c r="D15" s="11" t="n">
+      <c r="D15" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="E15" s="11" t="n">
+      <c r="E15" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="F15" s="11" t="n">
+      <c r="F15" s="14" t="n">
         <v>3.25</v>
       </c>
-      <c r="G15" s="11" t="n">
+      <c r="G15" s="14" t="n">
         <v>20</v>
       </c>
-      <c r="H15" s="11" t="n">
+      <c r="H15" s="14" t="n">
         <v>11.75</v>
       </c>
-      <c r="I15" s="11"/>
-      <c r="J15" s="11" t="n">
+      <c r="I15" s="14"/>
+      <c r="J15" s="14" t="n">
         <v>7</v>
       </c>
-      <c r="K15" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="L15" s="11" t="n">
+      <c r="K15" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="L15" s="14" t="n">
         <f aca="false">SUM(B15:K15)</f>
         <v>67.5</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="11" t="s">
+    <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="14" t="s">
         <v>92</v>
       </c>
-      <c r="B16" s="11" t="n">
+      <c r="B16" s="14" t="n">
         <v>39.5</v>
       </c>
-      <c r="C16" s="11" t="n">
+      <c r="C16" s="14" t="n">
         <v>8</v>
       </c>
-      <c r="D16" s="11"/>
-      <c r="E16" s="11"/>
-      <c r="F16" s="11" t="n">
+      <c r="D16" s="14"/>
+      <c r="E16" s="14"/>
+      <c r="F16" s="14" t="n">
         <v>4.5</v>
       </c>
-      <c r="G16" s="11"/>
-      <c r="H16" s="11" t="n">
+      <c r="G16" s="14"/>
+      <c r="H16" s="14" t="n">
         <v>7.25</v>
       </c>
-      <c r="I16" s="11"/>
-      <c r="J16" s="11"/>
-      <c r="K16" s="11" t="n">
+      <c r="I16" s="14"/>
+      <c r="J16" s="14"/>
+      <c r="K16" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="L16" s="11" t="n">
+      <c r="L16" s="14" t="n">
         <f aca="false">SUM(B16:K16)</f>
         <v>63.25</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="11" t="s">
+    <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="14" t="s">
         <v>88</v>
       </c>
-      <c r="B17" s="11" t="n">
+      <c r="B17" s="14" t="n">
+        <f aca="false">3+11</f>
+        <v>14</v>
+      </c>
+      <c r="C17" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="D17" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="E17" s="14" t="n">
+        <v>16.75</v>
+      </c>
+      <c r="F17" s="14" t="n">
+        <f aca="false">1+1</f>
+        <v>2</v>
+      </c>
+      <c r="G17" s="14" t="n">
+        <f aca="false">17.75+29</f>
+        <v>46.75</v>
+      </c>
+      <c r="H17" s="14" t="n">
+        <f aca="false">2+7</f>
+        <v>9</v>
+      </c>
+      <c r="I17" s="14"/>
+      <c r="J17" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="C17" s="11" t="n">
-        <v>4</v>
-      </c>
-      <c r="D17" s="11"/>
-      <c r="E17" s="11" t="n">
-        <v>16.75</v>
-      </c>
-      <c r="F17" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="G17" s="11" t="n">
-        <v>17.75</v>
-      </c>
-      <c r="H17" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="I17" s="11"/>
-      <c r="J17" s="11" t="n">
+      <c r="K17" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="L17" s="14" t="n">
+        <f aca="false">SUM(B17:K17)</f>
+        <v>104.5</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="14" t="s">
+        <v>87</v>
+      </c>
+      <c r="B18" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="C18" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="D18" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="E18" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="F18" s="14"/>
+      <c r="G18" s="14" t="n">
+        <v>7</v>
+      </c>
+      <c r="H18" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="K17" s="11" t="n">
-        <v>5</v>
-      </c>
-      <c r="L17" s="11" t="n">
-        <f aca="false">SUM(B17:K17)</f>
-        <v>52.5</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="11" t="s">
-        <v>87</v>
-      </c>
-      <c r="B18" s="11" t="n">
-        <v>5</v>
-      </c>
-      <c r="C18" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="D18" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="E18" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="F18" s="11"/>
-      <c r="G18" s="11" t="n">
-        <v>7</v>
-      </c>
-      <c r="H18" s="11" t="n">
-        <v>3</v>
-      </c>
-      <c r="I18" s="11"/>
-      <c r="J18" s="11" t="n">
+      <c r="I18" s="14"/>
+      <c r="J18" s="14" t="n">
         <v>17.5</v>
       </c>
-      <c r="K18" s="11" t="n">
+      <c r="K18" s="14" t="n">
         <v>4.5</v>
       </c>
-      <c r="L18" s="11" t="n">
+      <c r="L18" s="14" t="n">
         <f aca="false">SUM(B18:K18)</f>
         <v>40</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="11" t="s">
+    <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="14" t="s">
         <v>93</v>
       </c>
-      <c r="B19" s="11" t="n">
+      <c r="B19" s="14" t="n">
         <v>4.5</v>
       </c>
-      <c r="C19" s="11" t="n">
+      <c r="C19" s="14" t="n">
         <v>10.5</v>
       </c>
-      <c r="D19" s="11" t="n">
+      <c r="D19" s="14" t="n">
         <v>8.75</v>
       </c>
-      <c r="E19" s="11"/>
-      <c r="F19" s="11" t="n">
+      <c r="E19" s="14"/>
+      <c r="F19" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="G19" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="H19" s="11"/>
-      <c r="I19" s="11"/>
-      <c r="J19" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="K19" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="L19" s="11" t="n">
+      <c r="G19" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="H19" s="14"/>
+      <c r="I19" s="14"/>
+      <c r="J19" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="K19" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="L19" s="14" t="n">
         <f aca="false">SUM(B19:K19)</f>
         <v>33.75</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="11" t="s">
+    <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="14" t="s">
         <v>95</v>
       </c>
-      <c r="B20" s="11" t="n">
+      <c r="B20" s="14" t="n">
         <v>12</v>
       </c>
-      <c r="C20" s="11"/>
-      <c r="D20" s="11"/>
-      <c r="E20" s="11"/>
-      <c r="F20" s="11"/>
-      <c r="G20" s="11"/>
-      <c r="H20" s="11" t="n">
+      <c r="C20" s="14"/>
+      <c r="D20" s="14"/>
+      <c r="E20" s="14"/>
+      <c r="F20" s="14"/>
+      <c r="G20" s="14"/>
+      <c r="H20" s="14" t="n">
         <v>9.75</v>
       </c>
-      <c r="I20" s="11" t="n">
+      <c r="I20" s="14" t="n">
         <v>11</v>
       </c>
-      <c r="J20" s="11"/>
-      <c r="K20" s="11" t="n">
+      <c r="J20" s="14"/>
+      <c r="K20" s="14" t="n">
         <v>0.25</v>
       </c>
-      <c r="L20" s="11" t="n">
+      <c r="L20" s="14" t="n">
         <f aca="false">SUM(B20:K20)</f>
         <v>33</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="11" t="s">
+    <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="14" t="s">
         <v>97</v>
       </c>
-      <c r="B21" s="11"/>
-      <c r="C21" s="11"/>
-      <c r="D21" s="11" t="n">
+      <c r="B21" s="14"/>
+      <c r="C21" s="14"/>
+      <c r="D21" s="14" t="n">
         <v>24.25</v>
       </c>
-      <c r="E21" s="11"/>
-      <c r="F21" s="11"/>
-      <c r="G21" s="11" t="n">
+      <c r="E21" s="14"/>
+      <c r="F21" s="14"/>
+      <c r="G21" s="14" t="n">
         <v>8</v>
       </c>
-      <c r="H21" s="11"/>
-      <c r="I21" s="11"/>
-      <c r="J21" s="11"/>
-      <c r="K21" s="11"/>
-      <c r="L21" s="11" t="n">
+      <c r="H21" s="14"/>
+      <c r="I21" s="14"/>
+      <c r="J21" s="14"/>
+      <c r="K21" s="14"/>
+      <c r="L21" s="14" t="n">
         <f aca="false">SUM(B21:K21)</f>
         <v>32.25</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="11" t="s">
+    <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="14" t="s">
         <v>94</v>
       </c>
-      <c r="B22" s="11"/>
-      <c r="C22" s="11"/>
-      <c r="D22" s="11" t="n">
+      <c r="B22" s="14"/>
+      <c r="C22" s="14"/>
+      <c r="D22" s="14" t="n">
         <v>13</v>
       </c>
-      <c r="E22" s="11"/>
-      <c r="F22" s="11"/>
-      <c r="G22" s="11" t="n">
+      <c r="E22" s="14"/>
+      <c r="F22" s="14"/>
+      <c r="G22" s="14" t="n">
         <v>11</v>
       </c>
-      <c r="H22" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="I22" s="11"/>
-      <c r="J22" s="11" t="n">
+      <c r="H22" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="I22" s="14"/>
+      <c r="J22" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="K22" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="L22" s="11" t="n">
+      <c r="K22" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="L22" s="14" t="n">
         <f aca="false">SUM(B22:K22)</f>
         <v>31</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="11" t="s">
+    <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="14" t="s">
         <v>90</v>
       </c>
-      <c r="B23" s="11"/>
-      <c r="C23" s="11" t="n">
+      <c r="B23" s="14"/>
+      <c r="C23" s="14" t="n">
         <v>3.5</v>
       </c>
-      <c r="D23" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="E23" s="11"/>
-      <c r="F23" s="11" t="n">
+      <c r="D23" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="E23" s="14"/>
+      <c r="F23" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="G23" s="11" t="n">
+      <c r="G23" s="14" t="n">
         <v>1.5</v>
       </c>
-      <c r="H23" s="11" t="n">
+      <c r="H23" s="14" t="n">
         <v>13</v>
       </c>
-      <c r="I23" s="11"/>
-      <c r="J23" s="11" t="n">
+      <c r="I23" s="14"/>
+      <c r="J23" s="14" t="n">
         <v>1.75</v>
       </c>
-      <c r="K23" s="11" t="n">
+      <c r="K23" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="L23" s="11" t="n">
+      <c r="L23" s="14" t="n">
         <f aca="false">SUM(B23:K23)</f>
         <v>25.75</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="11" t="s">
+    <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="14" t="s">
         <v>96</v>
       </c>
-      <c r="B24" s="11"/>
-      <c r="C24" s="11"/>
-      <c r="D24" s="11"/>
-      <c r="E24" s="11"/>
-      <c r="F24" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="G24" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="H24" s="11"/>
-      <c r="I24" s="11"/>
-      <c r="J24" s="11"/>
-      <c r="K24" s="11" t="n">
+      <c r="B24" s="14"/>
+      <c r="C24" s="14"/>
+      <c r="D24" s="14"/>
+      <c r="E24" s="14"/>
+      <c r="F24" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="G24" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="H24" s="14"/>
+      <c r="I24" s="14"/>
+      <c r="J24" s="14"/>
+      <c r="K24" s="14" t="n">
         <v>10</v>
       </c>
-      <c r="L24" s="11" t="n">
+      <c r="L24" s="14" t="n">
         <f aca="false">SUM(B24:K24)</f>
         <v>12</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="11" t="s">
+    <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="14" t="s">
         <v>98</v>
       </c>
-      <c r="B25" s="11"/>
-      <c r="C25" s="11" t="n">
+      <c r="B25" s="14"/>
+      <c r="C25" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="D25" s="11" t="n">
+      <c r="D25" s="14" t="n">
         <v>6.5</v>
       </c>
-      <c r="E25" s="11"/>
-      <c r="F25" s="11"/>
-      <c r="G25" s="11"/>
-      <c r="H25" s="11"/>
-      <c r="I25" s="11"/>
-      <c r="J25" s="11"/>
-      <c r="K25" s="11"/>
-      <c r="L25" s="11" t="n">
+      <c r="E25" s="14"/>
+      <c r="F25" s="14"/>
+      <c r="G25" s="14"/>
+      <c r="H25" s="14"/>
+      <c r="I25" s="14"/>
+      <c r="J25" s="14"/>
+      <c r="K25" s="14"/>
+      <c r="L25" s="14" t="n">
         <f aca="false">SUM(B25:K25)</f>
         <v>11.5</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="11" t="s">
+    <row r="26" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="14" t="s">
         <v>99</v>
       </c>
-      <c r="B26" s="11"/>
-      <c r="C26" s="11"/>
-      <c r="D26" s="11"/>
-      <c r="E26" s="11"/>
-      <c r="F26" s="11"/>
-      <c r="G26" s="11"/>
-      <c r="H26" s="11"/>
-      <c r="I26" s="11" t="n">
+      <c r="B26" s="14"/>
+      <c r="C26" s="14"/>
+      <c r="D26" s="14"/>
+      <c r="E26" s="14"/>
+      <c r="F26" s="14"/>
+      <c r="G26" s="14"/>
+      <c r="H26" s="14"/>
+      <c r="I26" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="J26" s="11" t="n">
+      <c r="J26" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="K26" s="11"/>
-      <c r="L26" s="11" t="n">
+      <c r="K26" s="14"/>
+      <c r="L26" s="14" t="n">
         <f aca="false">SUM(B26:K26)</f>
         <v>10</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="11" t="s">
+    <row r="27" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="14" t="s">
         <v>100</v>
       </c>
-      <c r="B27" s="11"/>
-      <c r="C27" s="11"/>
-      <c r="D27" s="11"/>
-      <c r="E27" s="11"/>
-      <c r="F27" s="11"/>
-      <c r="G27" s="11"/>
-      <c r="H27" s="11"/>
-      <c r="I27" s="11"/>
-      <c r="J27" s="11"/>
-      <c r="K27" s="11" t="n">
+      <c r="B27" s="14"/>
+      <c r="C27" s="14"/>
+      <c r="D27" s="14"/>
+      <c r="E27" s="14"/>
+      <c r="F27" s="14"/>
+      <c r="G27" s="14"/>
+      <c r="H27" s="14"/>
+      <c r="I27" s="14"/>
+      <c r="J27" s="14"/>
+      <c r="K27" s="14" t="n">
         <v>3.5</v>
       </c>
-      <c r="L27" s="11" t="n">
+      <c r="L27" s="14" t="n">
         <f aca="false">SUM(B27:K27)</f>
         <v>3.5</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="7" t="s">
+    <row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="14" t="s">
+        <v>101</v>
+      </c>
+      <c r="B28" s="14" t="n">
+        <v>73</v>
+      </c>
+      <c r="C28" s="14" t="n">
+        <v>241</v>
+      </c>
+      <c r="D28" s="14" t="n">
+        <v>209</v>
+      </c>
+      <c r="E28" s="14" t="n">
+        <v>88</v>
+      </c>
+      <c r="F28" s="14" t="n">
+        <v>59</v>
+      </c>
+      <c r="G28" s="14" t="n">
+        <v>121</v>
+      </c>
+      <c r="H28" s="14" t="n">
+        <v>22</v>
+      </c>
+      <c r="I28" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="J28" s="14" t="n">
+        <v>28</v>
+      </c>
+      <c r="K28" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="L28" s="14" t="n">
+        <f aca="false">SUM(B28:K28)</f>
+        <v>846</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="7" t="s">
         <v>74</v>
       </c>
-      <c r="B28" s="7" t="n">
-        <f aca="false">SUM(B4:B27)</f>
-        <v>675.5</v>
-      </c>
-      <c r="C28" s="7" t="n">
-        <f aca="false">SUM(C4:C27)</f>
-        <v>627.25</v>
-      </c>
-      <c r="D28" s="7" t="n">
-        <f aca="false">SUM(D4:D27)</f>
-        <v>578.25</v>
-      </c>
-      <c r="E28" s="7" t="n">
-        <f aca="false">SUM(E4:E27)</f>
-        <v>572.05</v>
-      </c>
-      <c r="F28" s="7" t="n">
-        <f aca="false">SUM(F4:F27)</f>
-        <v>587.25</v>
-      </c>
-      <c r="G28" s="7" t="n">
-        <f aca="false">SUM(G4:G27)</f>
-        <v>668.3</v>
-      </c>
-      <c r="H28" s="7" t="n">
-        <f aca="false">SUM(H4:H27)</f>
-        <v>660.9</v>
-      </c>
-      <c r="I28" s="7" t="n">
-        <f aca="false">SUM(I4:I27)</f>
+      <c r="B29" s="7" t="n">
+        <f aca="false">SUM(B4:B28)</f>
+        <v>780.5</v>
+      </c>
+      <c r="C29" s="7" t="n">
+        <f aca="false">SUM(C4:C28)</f>
+        <v>872.25</v>
+      </c>
+      <c r="D29" s="7" t="n">
+        <f aca="false">SUM(D4:D28)</f>
+        <v>824.25</v>
+      </c>
+      <c r="E29" s="7" t="n">
+        <f aca="false">SUM(E4:E28)</f>
+        <v>673.05</v>
+      </c>
+      <c r="F29" s="7" t="n">
+        <f aca="false">SUM(F4:F28)</f>
+        <v>694.25</v>
+      </c>
+      <c r="G29" s="7" t="n">
+        <f aca="false">SUM(G4:G28)</f>
+        <v>837.3</v>
+      </c>
+      <c r="H29" s="7" t="n">
+        <f aca="false">SUM(H4:H28)</f>
+        <v>712.9</v>
+      </c>
+      <c r="I29" s="7" t="n">
+        <f aca="false">SUM(I4:I28)</f>
         <v>437.25</v>
       </c>
-      <c r="J28" s="7" t="n">
-        <f aca="false">SUM(J4:J27)</f>
-        <v>726.25</v>
-      </c>
-      <c r="K28" s="7" t="n">
-        <f aca="false">SUM(K4:K27)</f>
-        <v>385.25</v>
-      </c>
-      <c r="L28" s="7" t="n">
-        <f aca="false">SUM(L4:L27)</f>
-        <v>5918.25</v>
+      <c r="J29" s="7" t="n">
+        <f aca="false">SUM(J4:J28)</f>
+        <v>755.25</v>
+      </c>
+      <c r="K29" s="7" t="n">
+        <f aca="false">SUM(K4:K28)</f>
+        <v>390.25</v>
+      </c>
+      <c r="L29" s="7" t="n">
+        <f aca="false">SUM(L4:L28)</f>
+        <v>6977.25</v>
       </c>
     </row>
   </sheetData>
@@ -3617,29 +3829,29 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:L10"/>
-  <sheetFormatPr defaultColWidth="8.66796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.66796875" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="2" style="0" width="14"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="10" t="s">
-        <v>102</v>
-      </c>
-      <c r="B1" s="10"/>
-      <c r="C1" s="10"/>
-      <c r="D1" s="10"/>
-      <c r="E1" s="10"/>
-      <c r="F1" s="10"/>
-      <c r="G1" s="10"/>
-      <c r="H1" s="10"/>
-      <c r="I1" s="10"/>
-      <c r="J1" s="10"/>
-      <c r="K1" s="10"/>
-      <c r="L1" s="10"/>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="15" t="s">
+        <v>103</v>
+      </c>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="15"/>
+      <c r="G1" s="15"/>
+      <c r="H1" s="15"/>
+      <c r="I1" s="15"/>
+      <c r="J1" s="15"/>
+      <c r="K1" s="15"/>
+      <c r="L1" s="15"/>
+    </row>
+    <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
         <v>41</v>
       </c>
@@ -3677,215 +3889,215 @@
         <v>59</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="11" t="s">
-        <v>103</v>
-      </c>
-      <c r="B4" s="11" t="n">
+    <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="16" t="s">
+        <v>104</v>
+      </c>
+      <c r="B4" s="16" t="n">
         <v>77</v>
       </c>
-      <c r="C4" s="11" t="n">
+      <c r="C4" s="16" t="n">
         <v>73</v>
       </c>
-      <c r="D4" s="11" t="n">
+      <c r="D4" s="16" t="n">
         <v>66</v>
       </c>
-      <c r="E4" s="11" t="n">
+      <c r="E4" s="16" t="n">
         <v>57</v>
       </c>
-      <c r="F4" s="11" t="n">
+      <c r="F4" s="16" t="n">
         <v>87</v>
       </c>
-      <c r="G4" s="11" t="n">
+      <c r="G4" s="16" t="n">
         <v>97</v>
       </c>
-      <c r="H4" s="11" t="n">
+      <c r="H4" s="16" t="n">
         <v>106</v>
       </c>
-      <c r="I4" s="11" t="n">
+      <c r="I4" s="16" t="n">
         <v>25</v>
       </c>
-      <c r="J4" s="11" t="n">
+      <c r="J4" s="16" t="n">
         <v>76</v>
       </c>
-      <c r="K4" s="11" t="n">
+      <c r="K4" s="16" t="n">
         <v>87</v>
       </c>
-      <c r="L4" s="11" t="n">
+      <c r="L4" s="16" t="n">
         <f aca="false">SUM(B4:K4)</f>
         <v>751</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="11" t="s">
-        <v>104</v>
-      </c>
-      <c r="B5" s="11" t="n">
+    <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="16" t="s">
+        <v>105</v>
+      </c>
+      <c r="B5" s="16" t="n">
         <v>27</v>
       </c>
-      <c r="C5" s="11" t="n">
+      <c r="C5" s="16" t="n">
         <v>14</v>
       </c>
-      <c r="D5" s="11" t="n">
+      <c r="D5" s="16" t="n">
         <v>18</v>
       </c>
-      <c r="E5" s="11" t="n">
+      <c r="E5" s="16" t="n">
         <v>15</v>
       </c>
-      <c r="F5" s="11" t="n">
+      <c r="F5" s="16" t="n">
         <v>10</v>
       </c>
-      <c r="G5" s="11" t="n">
+      <c r="G5" s="16" t="n">
         <v>36</v>
       </c>
-      <c r="H5" s="11" t="n">
+      <c r="H5" s="16" t="n">
         <v>12</v>
       </c>
-      <c r="I5" s="11" t="n">
+      <c r="I5" s="16" t="n">
         <v>3</v>
       </c>
-      <c r="J5" s="11" t="n">
+      <c r="J5" s="16" t="n">
         <v>9</v>
       </c>
-      <c r="K5" s="11" t="n">
+      <c r="K5" s="16" t="n">
         <v>11</v>
       </c>
-      <c r="L5" s="11" t="n">
+      <c r="L5" s="16" t="n">
         <f aca="false">SUM(B5:K5)</f>
         <v>155</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="11" t="s">
-        <v>105</v>
-      </c>
-      <c r="B6" s="11" t="n">
+    <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="16" t="s">
+        <v>106</v>
+      </c>
+      <c r="B6" s="16" t="n">
         <v>4</v>
       </c>
-      <c r="C6" s="11" t="n">
+      <c r="C6" s="16" t="n">
         <v>13</v>
       </c>
-      <c r="D6" s="11" t="n">
+      <c r="D6" s="16" t="n">
         <v>4</v>
       </c>
-      <c r="E6" s="11" t="n">
+      <c r="E6" s="16" t="n">
         <v>16</v>
       </c>
-      <c r="F6" s="11" t="n">
+      <c r="F6" s="16" t="n">
         <v>13</v>
       </c>
-      <c r="G6" s="11" t="n">
+      <c r="G6" s="16" t="n">
         <v>13</v>
       </c>
-      <c r="H6" s="11" t="n">
+      <c r="H6" s="16" t="n">
         <v>13</v>
       </c>
-      <c r="I6" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="J6" s="11" t="n">
+      <c r="I6" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="J6" s="16" t="n">
         <v>24</v>
       </c>
-      <c r="K6" s="11" t="n">
+      <c r="K6" s="16" t="n">
         <v>36</v>
       </c>
-      <c r="L6" s="11" t="n">
+      <c r="L6" s="16" t="n">
         <f aca="false">SUM(B6:K6)</f>
         <v>138</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="11" t="s">
-        <v>106</v>
-      </c>
-      <c r="B7" s="11"/>
-      <c r="C7" s="11" t="n">
+    <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="16" t="s">
+        <v>107</v>
+      </c>
+      <c r="B7" s="16"/>
+      <c r="C7" s="16" t="n">
         <v>5</v>
       </c>
-      <c r="D7" s="11" t="n">
+      <c r="D7" s="16" t="n">
         <v>3</v>
       </c>
-      <c r="E7" s="11"/>
-      <c r="F7" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="G7" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="H7" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="I7" s="11"/>
-      <c r="J7" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="K7" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="L7" s="11" t="n">
+      <c r="E7" s="16"/>
+      <c r="F7" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="G7" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="H7" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="I7" s="16"/>
+      <c r="J7" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="K7" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="L7" s="16" t="n">
         <f aca="false">SUM(B7:K7)</f>
         <v>13</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="11" t="s">
-        <v>107</v>
-      </c>
-      <c r="B8" s="11"/>
-      <c r="C8" s="11"/>
-      <c r="D8" s="11"/>
-      <c r="E8" s="11"/>
-      <c r="F8" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="G8" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="H8" s="11" t="n">
+    <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="16" t="s">
+        <v>108</v>
+      </c>
+      <c r="B8" s="16"/>
+      <c r="C8" s="16"/>
+      <c r="D8" s="16"/>
+      <c r="E8" s="16"/>
+      <c r="F8" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="G8" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="H8" s="16" t="n">
         <v>4</v>
       </c>
-      <c r="I8" s="11"/>
-      <c r="J8" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="K8" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="L8" s="11" t="n">
+      <c r="I8" s="16"/>
+      <c r="J8" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="K8" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="L8" s="16" t="n">
         <f aca="false">SUM(B8:K8)</f>
         <v>10</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="11" t="s">
-        <v>108</v>
-      </c>
-      <c r="B9" s="11" t="n">
+    <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="16" t="s">
+        <v>109</v>
+      </c>
+      <c r="B9" s="16" t="n">
         <v>3</v>
       </c>
-      <c r="C9" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="D9" s="11"/>
-      <c r="E9" s="11"/>
-      <c r="F9" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="G9" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="H9" s="11"/>
-      <c r="I9" s="11"/>
-      <c r="J9" s="11"/>
-      <c r="K9" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="L9" s="11" t="n">
+      <c r="C9" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="D9" s="16"/>
+      <c r="E9" s="16"/>
+      <c r="F9" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="G9" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="H9" s="16"/>
+      <c r="I9" s="16"/>
+      <c r="J9" s="16"/>
+      <c r="K9" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="L9" s="16" t="n">
         <f aca="false">SUM(B9:K9)</f>
         <v>10</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
         <v>74</v>
       </c>
@@ -3954,7 +4166,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:K6"/>
-  <sheetFormatPr defaultColWidth="8.66796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.66796875" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="28"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="2" style="0" width="14"/>
@@ -3962,7 +4174,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="10" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B1" s="10"/>
       <c r="C1" s="10"/>
@@ -3975,9 +4187,9 @@
       <c r="J1" s="10"/>
       <c r="K1" s="10"/>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B3" s="7" t="s">
         <v>49</v>
@@ -4010,73 +4222,81 @@
         <v>58</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="13" t="s">
-        <v>111</v>
-      </c>
-      <c r="B4" s="11" t="n">
+    <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="17" t="s">
+        <v>112</v>
+      </c>
+      <c r="B4" s="14" t="n">
         <v>2.03</v>
       </c>
-      <c r="C4" s="11" t="n">
+      <c r="C4" s="14" t="n">
         <v>2.38</v>
       </c>
-      <c r="D4" s="11" t="n">
+      <c r="D4" s="14" t="n">
         <v>2.35</v>
       </c>
-      <c r="E4" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="F4" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="G4" s="11"/>
-      <c r="H4" s="11"/>
-      <c r="I4" s="11"/>
-      <c r="J4" s="11"/>
-      <c r="K4" s="11"/>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="13" t="s">
-        <v>112</v>
-      </c>
-      <c r="B5" s="11" t="n">
-        <v>2.06</v>
-      </c>
-      <c r="C5" s="11" t="n">
-        <v>1.84</v>
-      </c>
-      <c r="D5" s="11" t="n">
-        <v>1.63</v>
-      </c>
-      <c r="E5" s="11" t="n">
+      <c r="E4" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="F4" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="G4" s="14"/>
+      <c r="H4" s="14"/>
+      <c r="I4" s="14"/>
+      <c r="J4" s="14"/>
+      <c r="K4" s="14"/>
+    </row>
+    <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="17" t="s">
+        <v>101</v>
+      </c>
+      <c r="B5" s="14" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="C5" s="14" t="n">
         <v>1.7</v>
       </c>
-      <c r="F5" s="11" t="n">
-        <v>1.6</v>
-      </c>
-      <c r="G5" s="11"/>
-      <c r="H5" s="11"/>
-      <c r="I5" s="11"/>
-      <c r="J5" s="11"/>
-      <c r="K5" s="11"/>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D5" s="14" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="E5" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="G5" s="14" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="H5" s="14" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="I5" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" s="14" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="K5" s="14"/>
+    </row>
+    <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
         <v>113</v>
       </c>
-      <c r="B6" s="14" t="n">
+      <c r="B6" s="18" t="n">
         <f aca="false">AVERAGE(B4:K5)</f>
-        <v>1.959</v>
-      </c>
-      <c r="C6" s="14"/>
-      <c r="D6" s="14"/>
-      <c r="E6" s="14"/>
-      <c r="F6" s="14"/>
-      <c r="G6" s="14"/>
-      <c r="H6" s="14"/>
-      <c r="I6" s="14"/>
-      <c r="J6" s="14"/>
-      <c r="K6" s="14"/>
+        <v>1.69</v>
+      </c>
+      <c r="C6" s="18"/>
+      <c r="D6" s="18"/>
+      <c r="E6" s="18"/>
+      <c r="F6" s="18"/>
+      <c r="G6" s="18"/>
+      <c r="H6" s="18"/>
+      <c r="I6" s="18"/>
+      <c r="J6" s="18"/>
+      <c r="K6" s="18"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -4099,7 +4319,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:L5"/>
-  <sheetFormatPr defaultColWidth="8.66796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.66796875" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="28"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="2" style="0" width="14"/>
@@ -4121,9 +4341,9 @@
       <c r="K1" s="10"/>
       <c r="L1" s="10"/>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B3" s="7" t="s">
         <v>49</v>
@@ -4159,82 +4379,93 @@
         <v>59</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="13" t="s">
+    <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="17" t="s">
         <v>115</v>
       </c>
-      <c r="B4" s="11" t="n">
-        <v>25</v>
-      </c>
-      <c r="C4" s="11" t="n">
+      <c r="B4" s="14" t="n">
+        <f aca="false">25+1</f>
+        <v>26</v>
+      </c>
+      <c r="C4" s="14" t="n">
         <v>21</v>
       </c>
-      <c r="D4" s="11" t="n">
-        <v>22</v>
-      </c>
-      <c r="E4" s="11" t="n">
+      <c r="D4" s="14" t="n">
+        <f aca="false">22+1</f>
+        <v>23</v>
+      </c>
+      <c r="E4" s="14" t="n">
         <v>7</v>
       </c>
-      <c r="F4" s="11" t="n">
+      <c r="F4" s="14" t="n">
         <v>19</v>
       </c>
-      <c r="G4" s="11" t="n">
-        <v>29</v>
-      </c>
-      <c r="H4" s="11" t="n">
-        <v>36</v>
-      </c>
-      <c r="I4" s="11" t="n">
+      <c r="G4" s="14" t="n">
+        <f aca="false">29+1</f>
+        <v>30</v>
+      </c>
+      <c r="H4" s="14" t="n">
+        <f aca="false">36+1</f>
+        <v>37</v>
+      </c>
+      <c r="I4" s="14" t="n">
         <v>7</v>
       </c>
-      <c r="J4" s="11" t="n">
-        <v>16</v>
-      </c>
-      <c r="K4" s="11" t="n">
-        <v>22</v>
-      </c>
-      <c r="L4" s="11" t="n">
+      <c r="J4" s="14" t="n">
+        <f aca="false">16+1</f>
+        <v>17</v>
+      </c>
+      <c r="K4" s="14" t="n">
+        <f aca="false">22+1</f>
+        <v>23</v>
+      </c>
+      <c r="L4" s="14" t="n">
         <f aca="false">SUM(B4:K4)</f>
-        <v>204</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="13" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="17" t="s">
         <v>116</v>
       </c>
-      <c r="B5" s="11" t="n">
-        <v>13.75</v>
-      </c>
-      <c r="C5" s="11" t="n">
+      <c r="B5" s="14" t="n">
+        <f aca="false">13.75+12</f>
+        <v>25.75</v>
+      </c>
+      <c r="C5" s="14" t="n">
         <v>23.25</v>
       </c>
-      <c r="D5" s="11" t="n">
-        <v>19</v>
-      </c>
-      <c r="E5" s="11" t="n">
+      <c r="D5" s="14" t="n">
+        <f aca="false">19+16</f>
+        <v>35</v>
+      </c>
+      <c r="E5" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="F5" s="11" t="n">
+      <c r="F5" s="14" t="n">
         <v>12.25</v>
       </c>
-      <c r="G5" s="11" t="n">
-        <v>14.55</v>
-      </c>
-      <c r="H5" s="11" t="n">
-        <v>30.6</v>
-      </c>
-      <c r="I5" s="11" t="n">
+      <c r="G5" s="14" t="n">
+        <f aca="false">14.55+1</f>
+        <v>15.55</v>
+      </c>
+      <c r="H5" s="14" t="n">
+        <f aca="false">30.6+7</f>
+        <v>37.6</v>
+      </c>
+      <c r="I5" s="14" t="n">
         <v>12.75</v>
       </c>
-      <c r="J5" s="11" t="n">
-        <v>22</v>
-      </c>
-      <c r="K5" s="11" t="n">
+      <c r="J5" s="14" t="n">
+        <f aca="false">22+1</f>
+        <v>23</v>
+      </c>
+      <c r="K5" s="14" t="n">
         <v>8.5</v>
       </c>
-      <c r="L5" s="11" t="n">
+      <c r="L5" s="14" t="n">
         <f aca="false">SUM(B5:K5)</f>
-        <v>161.65</v>
+        <v>198.65</v>
       </c>
     </row>
   </sheetData>
@@ -4257,7 +4488,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:L4"/>
-  <sheetFormatPr defaultColWidth="11.5078125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.5625" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="13"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="2" style="0" width="14"/>
@@ -4279,7 +4510,7 @@
       <c r="K1" s="10"/>
       <c r="L1" s="10"/>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="7"/>
       <c r="B3" s="7" t="s">
         <v>49</v>
@@ -4315,43 +4546,43 @@
         <v>59</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="11" t="s">
+    <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="14" t="s">
         <v>118</v>
       </c>
-      <c r="B4" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="C4" s="11" t="n">
+      <c r="B4" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="C4" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="D4" s="11" t="n">
+      <c r="D4" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="E4" s="11" t="n">
+      <c r="E4" s="14" t="n">
         <v>8</v>
       </c>
-      <c r="F4" s="11" t="n">
+      <c r="F4" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="G4" s="11" t="n">
+      <c r="G4" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="H4" s="11" t="n">
+      <c r="H4" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="I4" s="11" t="n">
+      <c r="I4" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="J4" s="11" t="n">
+      <c r="J4" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="K4" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="K4" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="L4" s="11" t="n">
+      <c r="L4" s="14" t="n">
         <f aca="false">SUM(B4:K4)</f>
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>